<commit_message>
Align main docs with GitHub clone flow and link the Jev experiment branch.
Also bring backward-compatible runner updates (optional API key, token usage logging) without changing the default Nimble workbook Config.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/nimble_classifier_workbook.xlsx
+++ b/nimble_classifier_workbook.xlsx
@@ -629,6 +629,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="17">
       <c r="A4" s="38" t="inlineStr">
         <is>
@@ -717,7 +718,7 @@
       </c>
       <c r="B11" s="40" t="inlineStr">
         <is>
-          <t>Written by the runner: raw model JSON per record.</t>
+          <t>Written by the runner: raw model JSON per record (and usage_json when the API returns token usage).</t>
         </is>
       </c>
     </row>
@@ -741,7 +742,7 @@
       </c>
       <c r="B13" s="42" t="inlineStr">
         <is>
-          <t>Written by the runner: run metadata.</t>
+          <t>Written by the runner: run metadata (includes token totals when the API returns usage).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Unify Nimble and Jev in one workbook with engine-prefixed outputs.
Add --engine presets, keep each engine's results for output_compare, and archive the duplicate Jev workbook.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/nimble_classifier_workbook.xlsx
+++ b/nimble_classifier_workbook.xlsx
@@ -13,10 +13,15 @@
     <sheet name="Labels" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Records" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Lists" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="output_Results" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="output_Raw" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="output_Summary" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="output_Run_info" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="output_nimble_Results" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="output_nimble_Raw" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="output_nimble_Summary" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="output_nimble_Run_info" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="output_jev_Results" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="output_jev_Raw" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="output_jev_Summary" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="output_jev_Run_info" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="output_compare" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -28,7 +33,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -129,6 +134,15 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -199,7 +213,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -326,6 +340,8 @@
       <alignment horizontal="general" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -608,272 +624,256 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="22" customWidth="1" style="16" min="1" max="1"/>
-    <col width="90" customWidth="1" style="16" min="2" max="2"/>
+    <col width="28" customWidth="1" style="16" min="1" max="1"/>
+    <col width="110" customWidth="1" style="16" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.35" customHeight="1" s="17">
-      <c r="A1" s="18" t="inlineStr">
-        <is>
-          <t>Nimble batch classifier - control workbook</t>
+      <c r="A1" s="46" t="inlineStr">
+        <is>
+          <t>Nimble / Jev batch classifier - control workbook</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" s="17">
-      <c r="A2" s="19" t="inlineStr">
-        <is>
-          <t>Define questions, labels and records here. A program reads this file, sends each record to Nimble (Ollama /v1/systemone), clears any existing output_* sheets, then writes fresh output_* sheets back into this same workbook.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>Define questions, labels and records here. Run with --engine nimble or --engine jev. Each engine writes its own output_&lt;engine&gt;_* sheets and does not clear the other. When both Results sheets exist, output_compare is refreshed.</t>
+        </is>
+      </c>
+    </row>
     <row r="4" ht="15" customHeight="1" s="17">
-      <c r="A4" s="38" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>SHEETS</t>
         </is>
       </c>
-      <c r="B4" s="21" t="n"/>
     </row>
     <row r="5" ht="15" customHeight="1" s="17">
-      <c r="A5" s="39" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Config</t>
         </is>
       </c>
-      <c r="B5" s="40" t="inlineStr">
-        <is>
-          <t>Settings: model, URL, timeout, default review threshold, test-run size.</t>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Settings: engine (nimble|jev), timeouts, review threshold, test-run size. Engine preset overrides model/base_url/endpoint.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" s="17">
-      <c r="A6" s="39" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>Questions</t>
         </is>
       </c>
-      <c r="B6" s="40" t="inlineStr">
-        <is>
-          <t>One row per question. Type is choice (pick one label), noul (yes/no) or score (place on a scale). Leave equipment_type blank to ask the question of every record.</t>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>One row per question. Type is choice, noul (yes/no) or score. Leave equipment_type blank to ask every record.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" s="17">
-      <c r="A7" s="39" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>Labels</t>
         </is>
       </c>
-      <c r="B7" s="40" t="inlineStr">
-        <is>
-          <t>One row per answer option, for choice and score questions only. noul questions take no labels. For score questions, 'order' is the position on the scale, lowest first.</t>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Answer options for choice and score only. For score, order is scale position (lowest first).</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1" s="17">
-      <c r="A8" s="39" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>Records</t>
         </is>
       </c>
-      <c r="B8" s="40" t="inlineStr">
-        <is>
-          <t>One row per statement to classify. Optional expected_&lt;question_id&gt; columns hold the known correct answer, so the program can measure accuracy.</t>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>Statements to classify. Optional expected_&lt;question_id&gt; columns for accuracy.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="17">
-      <c r="A9" s="39" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>Lists</t>
         </is>
       </c>
-      <c r="B9" s="40" t="inlineStr">
-        <is>
-          <t>Dropdown values (equipment types). Add new equipment types here.</t>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Dropdown values (equipment types).</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="17">
-      <c r="A10" s="41" t="inlineStr">
-        <is>
-          <t>output_Results</t>
-        </is>
-      </c>
-      <c r="B10" s="42" t="inlineStr">
-        <is>
-          <t>Written by the runner: answers, confidence, review flags. Cleared at the start of each run, rewritten when the run finishes.</t>
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>output_nimble_*</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Written by --engine nimble: Results, Raw, Summary, Run_info.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="17">
-      <c r="A11" s="39" t="inlineStr">
-        <is>
-          <t>output_Raw</t>
-        </is>
-      </c>
-      <c r="B11" s="40" t="inlineStr">
-        <is>
-          <t>Written by the runner: raw model JSON per record (and usage_json when the API returns token usage).</t>
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>output_jev_*</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Written by --engine jev: Results, Raw, Summary, Run_info.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="17">
-      <c r="A12" s="43" t="inlineStr">
-        <is>
-          <t>output_Summary</t>
-        </is>
-      </c>
-      <c r="B12" s="40" t="inlineStr">
-        <is>
-          <t>Written by the runner: accuracy / confidence stats (accuracy needs expected_* columns).</t>
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>output_compare</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Side-by-side Nimble vs Jev answers when both Results sheets exist. Diffs highlighted.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="17">
-      <c r="A13" s="41" t="inlineStr">
-        <is>
-          <t>output_Run_info</t>
-        </is>
-      </c>
-      <c r="B13" s="42" t="inlineStr">
-        <is>
-          <t>Written by the runner: run metadata (includes token totals when the API returns usage).</t>
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>COLOURS</t>
         </is>
       </c>
     </row>
     <row r="14" ht="45" customHeight="1" s="17">
-      <c r="A14" s="44" t="inlineStr">
-        <is>
-          <t>COLOURS</t>
-        </is>
-      </c>
-      <c r="B14" s="19" t="n"/>
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>Blue text</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>Cells you edit.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1" s="17">
-      <c r="A15" s="39" t="inlineStr">
-        <is>
-          <t>Blue text</t>
-        </is>
-      </c>
-      <c r="B15" s="40" t="inlineStr">
-        <is>
-          <t>Cells you edit.</t>
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>Black text, grey fill</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Formulas. Do not edit.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="17">
-      <c r="A16" s="39" t="inlineStr">
-        <is>
-          <t>Black text, grey fill</t>
-        </is>
-      </c>
-      <c r="B16" s="40" t="inlineStr">
-        <is>
-          <t>Formulas. Do not edit. The 'check' columns turn red when a row has a problem.</t>
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>Yellow row</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>Flagged for review (low confidence).</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1" s="17">
-      <c r="A17" s="44" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>Orange row (compare)</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Nimble and Jev answers disagree.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1" s="17">
+      <c r="A18" s="16" t="inlineStr">
         <is>
           <t>RULES</t>
         </is>
       </c>
-      <c r="B17" s="19" t="n"/>
-    </row>
-    <row r="18" ht="30" customHeight="1" s="17">
-      <c r="A18" s="39" t="inlineStr">
+    </row>
+    <row r="19" ht="30" customHeight="1" s="17">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>Engine</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Use Config engine or CLI --engine. Jev needs TYPESAFE_API_KEY. Nimble needs local Ollama &gt;= 0.35.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1" s="17">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>IDs</t>
         </is>
       </c>
-      <c r="B18" s="40" t="inlineStr">
-        <is>
-          <t>question_id and label values are sent to the model as keys. Use short lowercase words with underscores, no spaces or quotes (e.g. tube_leak). question_id must be unique across the whole workbook.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1" s="17">
-      <c r="A19" s="39" t="inlineStr">
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>question_id and label: short lowercase with underscores, no spaces.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="45" customHeight="1" s="17">
+      <c r="A21" s="16" t="inlineStr">
         <is>
           <t>Always add 'other'</t>
         </is>
       </c>
-      <c r="B19" s="40" t="inlineStr">
-        <is>
-          <t>Nimble can only pick from the labels you give it. Include an 'other' label on every choice question so vague records are not forced into a wrong category.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="15" customHeight="1" s="17">
-      <c r="A20" s="41" t="inlineStr">
-        <is>
-          <t>One idea per question</t>
-        </is>
-      </c>
-      <c r="B20" s="42" t="inlineStr">
-        <is>
-          <t>Ask about what the text says, not what only an engineer would infer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="45" customHeight="1" s="17">
-      <c r="A21" s="39" t="inlineStr">
-        <is>
-          <t>Equipment type</t>
-        </is>
-      </c>
-      <c r="B21" s="40" t="inlineStr">
-        <is>
-          <t>A record is asked every question whose equipment_type matches its own, plus every question with a blank equipment_type.</t>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Include other on every choice question.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="35" t="inlineStr">
+      <c r="A22" s="16" t="inlineStr">
         <is>
           <t>Expected values</t>
         </is>
       </c>
-      <c r="B22" s="40" t="inlineStr">
-        <is>
-          <t>For choice questions, use a label from the Labels sheet. For noul questions, use true or false. Leave blank if unknown.</t>
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>choice: a Labels value; noul: true or false.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="35" t="inlineStr">
-        <is>
-          <t>Thresholds</t>
-        </is>
-      </c>
-      <c r="B23" s="40" t="inlineStr">
-        <is>
-          <t>review_below is the confidence under which a row is flagged for a person to review. The default of 0.6 on Config is a placeholder: tune it using records with known answers.</t>
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>EXAMPLES</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="45" t="inlineStr">
-        <is>
-          <t>EXAMPLES</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="35" t="inlineStr">
+      <c r="A24" s="16" t="inlineStr">
         <is>
           <t>Example rows</t>
         </is>
       </c>
-      <c r="B25" s="40" t="inlineStr">
-        <is>
-          <t>The rows filled in on every sheet are illustrative examples for pumps, heat exchangers and distillation columns. The expected values are examples, not validated data. Replace or delete them.</t>
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>Illustrative pumps / exchangers / columns. Replace with your plant data.</t>
         </is>
       </c>
     </row>
@@ -893,7 +893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" style="17" min="1" max="1"/>
@@ -920,7 +920,7 @@
       </c>
       <c r="B2" s="35" t="inlineStr">
         <is>
-          <t>20260930_112907</t>
+          <t>20260930_142141</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
     <row r="4">
       <c r="A4" s="35" t="inlineStr">
         <is>
-          <t>model</t>
+          <t>engine</t>
         </is>
       </c>
       <c r="B4" s="35" t="inlineStr">
@@ -951,109 +951,2536 @@
     <row r="5">
       <c r="A5" s="35" t="inlineStr">
         <is>
-          <t>ollama_version</t>
+          <t>model</t>
         </is>
       </c>
       <c r="B5" s="35" t="inlineStr">
         <is>
-          <t>0.35.0</t>
+          <t>nimble</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="35" t="inlineStr">
         <is>
-          <t>questions_hash</t>
+          <t>base_url</t>
         </is>
       </c>
       <c r="B6" s="35" t="inlineStr">
         <is>
-          <t>f73a405167a3</t>
+          <t>http://localhost:11434</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>records_in_run</t>
+          <t>endpoint_info</t>
         </is>
       </c>
       <c r="B7" s="35" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0.35.0</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="35" t="inlineStr">
         <is>
-          <t>records_completed</t>
+          <t>questions_hash</t>
         </is>
       </c>
       <c r="B8" s="35" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>f73a405167a3</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="35" t="inlineStr">
         <is>
-          <t>failed_records</t>
+          <t>api_key_configured</t>
         </is>
       </c>
       <c r="B9" s="35" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>True</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="35" t="inlineStr">
         <is>
-          <t>review_threshold_default</t>
+          <t>records_in_run</t>
         </is>
       </c>
       <c r="B10" s="35" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>6</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="35" t="inlineStr">
         <is>
-          <t>elapsed_seconds</t>
+          <t>records_completed</t>
         </is>
       </c>
       <c r="B11" s="35" t="inlineStr">
         <is>
-          <t>42.8</t>
+          <t>6</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="35" t="inlineStr">
         <is>
-          <t>checkpoint</t>
+          <t>failed_records</t>
         </is>
       </c>
       <c r="B12" s="35" t="inlineStr">
         <is>
-          <t>/mnt/d/dev/nimble_plant/nimble_classifier_workbook_20260930_112907.jsonl</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="35" t="inlineStr">
         <is>
+          <t>review_threshold_default</t>
+        </is>
+      </c>
+      <c r="B13" s="35" t="inlineStr">
+        <is>
+          <t>0.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="35" t="inlineStr">
+        <is>
+          <t>elapsed_seconds</t>
+        </is>
+      </c>
+      <c r="B14" s="35" t="inlineStr">
+        <is>
+          <t>45.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="35" t="inlineStr">
+        <is>
+          <t>checkpoint</t>
+        </is>
+      </c>
+      <c r="B15" s="35" t="inlineStr">
+        <is>
+          <t>/mnt/d/dev/nimble_plant/nimble_classifier_workbook_nimble_20260930_142141.jsonl</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="35" t="inlineStr">
+        <is>
+          <t>input_tokens</t>
+        </is>
+      </c>
+      <c r="B16" s="35" t="inlineStr">
+        <is>
+          <t>6698</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="35" t="inlineStr">
+        <is>
+          <t>output_tokens</t>
+        </is>
+      </c>
+      <c r="B17" s="35" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="35" t="inlineStr">
+        <is>
+          <t>total_tokens</t>
+        </is>
+      </c>
+      <c r="B18" s="35" t="inlineStr">
+        <is>
+          <t>6722</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="35" t="inlineStr">
+        <is>
+          <t>records_with_usage</t>
+        </is>
+      </c>
+      <c r="B19" s="35" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="35" t="inlineStr">
+        <is>
           <t>output_sheets</t>
         </is>
       </c>
+      <c r="B20" s="35" t="inlineStr">
+        <is>
+          <t>output_nimble_Results, output_nimble_Raw, output_nimble_Summary, output_nimble_Run_info</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AH7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" style="17" min="1" max="1"/>
+    <col width="12" customWidth="1" style="17" min="2" max="2"/>
+    <col width="12" customWidth="1" style="17" min="3" max="3"/>
+    <col width="60" customWidth="1" style="17" min="4" max="4"/>
+    <col width="16" customWidth="1" style="17" min="5" max="5"/>
+    <col width="12" customWidth="1" style="17" min="6" max="6"/>
+    <col width="10" customWidth="1" style="17" min="7" max="7"/>
+    <col width="16" customWidth="1" style="17" min="8" max="8"/>
+    <col width="12" customWidth="1" style="17" min="9" max="9"/>
+    <col width="10" customWidth="1" style="17" min="10" max="10"/>
+    <col width="16" customWidth="1" style="17" min="11" max="11"/>
+    <col width="12" customWidth="1" style="17" min="12" max="12"/>
+    <col width="10" customWidth="1" style="17" min="13" max="13"/>
+    <col width="16" customWidth="1" style="17" min="14" max="14"/>
+    <col width="12" customWidth="1" style="17" min="15" max="15"/>
+    <col width="10" customWidth="1" style="17" min="16" max="16"/>
+    <col width="16" customWidth="1" style="17" min="17" max="17"/>
+    <col width="12" customWidth="1" style="17" min="18" max="18"/>
+    <col width="10" customWidth="1" style="17" min="19" max="19"/>
+    <col width="16" customWidth="1" style="17" min="20" max="20"/>
+    <col width="12" customWidth="1" style="17" min="21" max="21"/>
+    <col width="10" customWidth="1" style="17" min="22" max="22"/>
+    <col width="16" customWidth="1" style="17" min="23" max="23"/>
+    <col width="12" customWidth="1" style="17" min="24" max="24"/>
+    <col width="10" customWidth="1" style="17" min="25" max="25"/>
+    <col width="16" customWidth="1" style="17" min="26" max="26"/>
+    <col width="12" customWidth="1" style="17" min="27" max="27"/>
+    <col width="10" customWidth="1" style="17" min="28" max="28"/>
+    <col width="16" customWidth="1" style="17" min="29" max="29"/>
+    <col width="12" customWidth="1" style="17" min="30" max="30"/>
+    <col width="10" customWidth="1" style="17" min="31" max="31"/>
+    <col width="12" customWidth="1" style="17" min="32" max="32"/>
+    <col width="45" customWidth="1" style="17" min="33" max="33"/>
+    <col width="30" customWidth="1" style="17" min="34" max="34"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="31" t="inlineStr">
+        <is>
+          <t>record_id</t>
+        </is>
+      </c>
+      <c r="B1" s="31" t="inlineStr">
+        <is>
+          <t>equipment_type</t>
+        </is>
+      </c>
+      <c r="C1" s="31" t="inlineStr">
+        <is>
+          <t>tag</t>
+        </is>
+      </c>
+      <c r="D1" s="31" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E1" s="31" t="inlineStr">
+        <is>
+          <t>pump_failure_mode__answer</t>
+        </is>
+      </c>
+      <c r="F1" s="31" t="inlineStr">
+        <is>
+          <t>pump_failure_mode__confidence</t>
+        </is>
+      </c>
+      <c r="G1" s="31" t="inlineStr">
+        <is>
+          <t>pump_failure_mode__value</t>
+        </is>
+      </c>
+      <c r="H1" s="31" t="inlineStr">
+        <is>
+          <t>pump_containment__answer</t>
+        </is>
+      </c>
+      <c r="I1" s="31" t="inlineStr">
+        <is>
+          <t>pump_containment__confidence</t>
+        </is>
+      </c>
+      <c r="J1" s="31" t="inlineStr">
+        <is>
+          <t>pump_containment__value</t>
+        </is>
+      </c>
+      <c r="K1" s="31" t="inlineStr">
+        <is>
+          <t>pump_urgency__answer</t>
+        </is>
+      </c>
+      <c r="L1" s="31" t="inlineStr">
+        <is>
+          <t>pump_urgency__confidence</t>
+        </is>
+      </c>
+      <c r="M1" s="31" t="inlineStr">
+        <is>
+          <t>pump_urgency__value</t>
+        </is>
+      </c>
+      <c r="N1" s="31" t="inlineStr">
+        <is>
+          <t>hx_problem__answer</t>
+        </is>
+      </c>
+      <c r="O1" s="31" t="inlineStr">
+        <is>
+          <t>hx_problem__confidence</t>
+        </is>
+      </c>
+      <c r="P1" s="31" t="inlineStr">
+        <is>
+          <t>hx_problem__value</t>
+        </is>
+      </c>
+      <c r="Q1" s="31" t="inlineStr">
+        <is>
+          <t>hx_crosscontam__answer</t>
+        </is>
+      </c>
+      <c r="R1" s="31" t="inlineStr">
+        <is>
+          <t>hx_crosscontam__confidence</t>
+        </is>
+      </c>
+      <c r="S1" s="31" t="inlineStr">
+        <is>
+          <t>hx_crosscontam__value</t>
+        </is>
+      </c>
+      <c r="T1" s="31" t="inlineStr">
+        <is>
+          <t>hx_impact__answer</t>
+        </is>
+      </c>
+      <c r="U1" s="31" t="inlineStr">
+        <is>
+          <t>hx_impact__confidence</t>
+        </is>
+      </c>
+      <c r="V1" s="31" t="inlineStr">
+        <is>
+          <t>hx_impact__value</t>
+        </is>
+      </c>
+      <c r="W1" s="31" t="inlineStr">
+        <is>
+          <t>col_symptom__answer</t>
+        </is>
+      </c>
+      <c r="X1" s="31" t="inlineStr">
+        <is>
+          <t>col_symptom__confidence</t>
+        </is>
+      </c>
+      <c r="Y1" s="31" t="inlineStr">
+        <is>
+          <t>col_symptom__value</t>
+        </is>
+      </c>
+      <c r="Z1" s="31" t="inlineStr">
+        <is>
+          <t>col_offspec__answer</t>
+        </is>
+      </c>
+      <c r="AA1" s="31" t="inlineStr">
+        <is>
+          <t>col_offspec__confidence</t>
+        </is>
+      </c>
+      <c r="AB1" s="31" t="inlineStr">
+        <is>
+          <t>col_offspec__value</t>
+        </is>
+      </c>
+      <c r="AC1" s="31" t="inlineStr">
+        <is>
+          <t>col_stability__answer</t>
+        </is>
+      </c>
+      <c r="AD1" s="31" t="inlineStr">
+        <is>
+          <t>col_stability__confidence</t>
+        </is>
+      </c>
+      <c r="AE1" s="31" t="inlineStr">
+        <is>
+          <t>col_stability__value</t>
+        </is>
+      </c>
+      <c r="AF1" s="31" t="inlineStr">
+        <is>
+          <t>needs_review</t>
+        </is>
+      </c>
+      <c r="AG1" s="31" t="inlineStr">
+        <is>
+          <t>review_reasons</t>
+        </is>
+      </c>
+      <c r="AH1" s="31" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="35" t="inlineStr">
+        <is>
+          <t>R001</t>
+        </is>
+      </c>
+      <c r="B2" s="35" t="inlineStr">
+        <is>
+          <t>Pump</t>
+        </is>
+      </c>
+      <c r="C2" s="35" t="inlineStr">
+        <is>
+          <t>P-101A</t>
+        </is>
+      </c>
+      <c r="D2" s="36" t="inlineStr">
+        <is>
+          <t>P-101A discharge pressure fluctuating, seal leak observed, standby pump started.</t>
+        </is>
+      </c>
+      <c r="E2" s="35" t="inlineStr">
+        <is>
+          <t>seal</t>
+        </is>
+      </c>
+      <c r="F2" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="35" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I2" s="37" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J2" s="37" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="K2" s="35" t="inlineStr">
+        <is>
+          <t>immediate</t>
+        </is>
+      </c>
+      <c r="L2" s="37" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="M2" s="37" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="N2" s="35" t="inlineStr"/>
+      <c r="O2" s="35" t="inlineStr"/>
+      <c r="P2" s="35" t="inlineStr"/>
+      <c r="Q2" s="35" t="inlineStr"/>
+      <c r="R2" s="35" t="inlineStr"/>
+      <c r="S2" s="35" t="inlineStr"/>
+      <c r="T2" s="35" t="inlineStr"/>
+      <c r="U2" s="35" t="inlineStr"/>
+      <c r="V2" s="35" t="inlineStr"/>
+      <c r="W2" s="35" t="inlineStr"/>
+      <c r="X2" s="35" t="inlineStr"/>
+      <c r="Y2" s="35" t="inlineStr"/>
+      <c r="Z2" s="35" t="inlineStr"/>
+      <c r="AA2" s="35" t="inlineStr"/>
+      <c r="AB2" s="35" t="inlineStr"/>
+      <c r="AC2" s="35" t="inlineStr"/>
+      <c r="AD2" s="35" t="inlineStr"/>
+      <c r="AE2" s="35" t="inlineStr"/>
+      <c r="AF2" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="AG2" s="35" t="inlineStr"/>
+      <c r="AH2" s="35" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="35" t="inlineStr">
+        <is>
+          <t>R002</t>
+        </is>
+      </c>
+      <c r="B3" s="35" t="inlineStr">
+        <is>
+          <t>Pump</t>
+        </is>
+      </c>
+      <c r="C3" s="35" t="inlineStr">
+        <is>
+          <t>P-114</t>
+        </is>
+      </c>
+      <c r="D3" s="36" t="inlineStr">
+        <is>
+          <t>Routine check on P-114 shows slightly elevated bearing temperature. Watch at next planned PM.</t>
+        </is>
+      </c>
+      <c r="E3" s="35" t="inlineStr">
+        <is>
+          <t>bearing</t>
+        </is>
+      </c>
+      <c r="F3" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" s="35" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="I3" s="37" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J3" s="37" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K3" s="35" t="inlineStr">
+        <is>
+          <t>routine</t>
+        </is>
+      </c>
+      <c r="L3" s="37" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="M3" s="37" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="N3" s="35" t="inlineStr"/>
+      <c r="O3" s="35" t="inlineStr"/>
+      <c r="P3" s="35" t="inlineStr"/>
+      <c r="Q3" s="35" t="inlineStr"/>
+      <c r="R3" s="35" t="inlineStr"/>
+      <c r="S3" s="35" t="inlineStr"/>
+      <c r="T3" s="35" t="inlineStr"/>
+      <c r="U3" s="35" t="inlineStr"/>
+      <c r="V3" s="35" t="inlineStr"/>
+      <c r="W3" s="35" t="inlineStr"/>
+      <c r="X3" s="35" t="inlineStr"/>
+      <c r="Y3" s="35" t="inlineStr"/>
+      <c r="Z3" s="35" t="inlineStr"/>
+      <c r="AA3" s="35" t="inlineStr"/>
+      <c r="AB3" s="35" t="inlineStr"/>
+      <c r="AC3" s="35" t="inlineStr"/>
+      <c r="AD3" s="35" t="inlineStr"/>
+      <c r="AE3" s="35" t="inlineStr"/>
+      <c r="AF3" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="AG3" s="35" t="inlineStr"/>
+      <c r="AH3" s="35" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="35" t="inlineStr">
+        <is>
+          <t>R003</t>
+        </is>
+      </c>
+      <c r="B4" s="35" t="inlineStr">
+        <is>
+          <t>Heat Exchanger</t>
+        </is>
+      </c>
+      <c r="C4" s="35" t="inlineStr">
+        <is>
+          <t>E-205</t>
+        </is>
+      </c>
+      <c r="D4" s="36" t="inlineStr">
+        <is>
+          <t>E-205 outlet temperature 15 C below normal, dP up over last two weeks, cleaning scheduled.</t>
+        </is>
+      </c>
+      <c r="E4" s="35" t="inlineStr"/>
+      <c r="F4" s="35" t="inlineStr"/>
+      <c r="G4" s="35" t="inlineStr"/>
+      <c r="H4" s="35" t="inlineStr"/>
+      <c r="I4" s="35" t="inlineStr"/>
+      <c r="J4" s="35" t="inlineStr"/>
+      <c r="K4" s="35" t="inlineStr"/>
+      <c r="L4" s="35" t="inlineStr"/>
+      <c r="M4" s="35" t="inlineStr"/>
+      <c r="N4" s="35" t="inlineStr">
+        <is>
+          <t>fouling</t>
+        </is>
+      </c>
+      <c r="O4" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="P4" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q4" s="35" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="R4" s="37" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="S4" s="37" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="T4" s="35" t="inlineStr">
+        <is>
+          <t>degraded</t>
+        </is>
+      </c>
+      <c r="U4" s="37" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="V4" s="37" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="W4" s="35" t="inlineStr"/>
+      <c r="X4" s="35" t="inlineStr"/>
+      <c r="Y4" s="35" t="inlineStr"/>
+      <c r="Z4" s="35" t="inlineStr"/>
+      <c r="AA4" s="35" t="inlineStr"/>
+      <c r="AB4" s="35" t="inlineStr"/>
+      <c r="AC4" s="35" t="inlineStr"/>
+      <c r="AD4" s="35" t="inlineStr"/>
+      <c r="AE4" s="35" t="inlineStr"/>
+      <c r="AF4" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="AG4" s="35" t="inlineStr"/>
+      <c r="AH4" s="35" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="32" t="inlineStr">
+        <is>
+          <t>R004</t>
+        </is>
+      </c>
+      <c r="B5" s="32" t="inlineStr">
+        <is>
+          <t>Heat Exchanger</t>
+        </is>
+      </c>
+      <c r="C5" s="32" t="inlineStr">
+        <is>
+          <t>E-310</t>
+        </is>
+      </c>
+      <c r="D5" s="33" t="inlineStr">
+        <is>
+          <t>Cooling water pH dropped and hydrocarbon detected in E-310 cooling water return. Suspect tube leak.</t>
+        </is>
+      </c>
+      <c r="E5" s="32" t="inlineStr"/>
+      <c r="F5" s="32" t="inlineStr"/>
+      <c r="G5" s="32" t="inlineStr"/>
+      <c r="H5" s="32" t="inlineStr"/>
+      <c r="I5" s="32" t="inlineStr"/>
+      <c r="J5" s="32" t="inlineStr"/>
+      <c r="K5" s="32" t="inlineStr"/>
+      <c r="L5" s="32" t="inlineStr"/>
+      <c r="M5" s="32" t="inlineStr"/>
+      <c r="N5" s="32" t="inlineStr">
+        <is>
+          <t>tube_leak</t>
+        </is>
+      </c>
+      <c r="O5" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="P5" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q5" s="32" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="R5" s="34" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="S5" s="34" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="T5" s="32" t="inlineStr">
+        <is>
+          <t>degraded</t>
+        </is>
+      </c>
+      <c r="U5" s="34" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="V5" s="34" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="W5" s="32" t="inlineStr"/>
+      <c r="X5" s="32" t="inlineStr"/>
+      <c r="Y5" s="32" t="inlineStr"/>
+      <c r="Z5" s="32" t="inlineStr"/>
+      <c r="AA5" s="32" t="inlineStr"/>
+      <c r="AB5" s="32" t="inlineStr"/>
+      <c r="AC5" s="32" t="inlineStr"/>
+      <c r="AD5" s="32" t="inlineStr"/>
+      <c r="AE5" s="32" t="inlineStr"/>
+      <c r="AF5" s="32" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG5" s="32" t="inlineStr">
+        <is>
+          <t>hx_impact: low confidence (0.49)</t>
+        </is>
+      </c>
+      <c r="AH5" s="32" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="35" t="inlineStr">
+        <is>
+          <t>R005</t>
+        </is>
+      </c>
+      <c r="B6" s="35" t="inlineStr">
+        <is>
+          <t>Distillation Column</t>
+        </is>
+      </c>
+      <c r="C6" s="35" t="inlineStr">
+        <is>
+          <t>C-301</t>
+        </is>
+      </c>
+      <c r="D6" s="36" t="inlineStr">
+        <is>
+          <t>C-301 dP spiking, bottoms level unstable, overhead product off-spec since 14:20.</t>
+        </is>
+      </c>
+      <c r="E6" s="35" t="inlineStr"/>
+      <c r="F6" s="35" t="inlineStr"/>
+      <c r="G6" s="35" t="inlineStr"/>
+      <c r="H6" s="35" t="inlineStr"/>
+      <c r="I6" s="35" t="inlineStr"/>
+      <c r="J6" s="35" t="inlineStr"/>
+      <c r="K6" s="35" t="inlineStr"/>
+      <c r="L6" s="35" t="inlineStr"/>
+      <c r="M6" s="35" t="inlineStr"/>
+      <c r="N6" s="35" t="inlineStr"/>
+      <c r="O6" s="35" t="inlineStr"/>
+      <c r="P6" s="35" t="inlineStr"/>
+      <c r="Q6" s="35" t="inlineStr"/>
+      <c r="R6" s="35" t="inlineStr"/>
+      <c r="S6" s="35" t="inlineStr"/>
+      <c r="T6" s="35" t="inlineStr"/>
+      <c r="U6" s="35" t="inlineStr"/>
+      <c r="V6" s="35" t="inlineStr"/>
+      <c r="W6" s="35" t="inlineStr">
+        <is>
+          <t>flooding</t>
+        </is>
+      </c>
+      <c r="X6" s="37" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="Y6" s="37" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="Z6" s="35" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AA6" s="37" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="AB6" s="37" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="AC6" s="35" t="inlineStr">
+        <is>
+          <t>upset</t>
+        </is>
+      </c>
+      <c r="AD6" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE6" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="AF6" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="AG6" s="35" t="inlineStr"/>
+      <c r="AH6" s="35" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="35" t="inlineStr">
+        <is>
+          <t>R006</t>
+        </is>
+      </c>
+      <c r="B7" s="35" t="inlineStr">
+        <is>
+          <t>Distillation Column</t>
+        </is>
+      </c>
+      <c r="C7" s="35" t="inlineStr">
+        <is>
+          <t>C-402</t>
+        </is>
+      </c>
+      <c r="D7" s="36" t="inlineStr">
+        <is>
+          <t>C-402 running steady at rate. Reflux and reboiler duty normal, no alarms this shift.</t>
+        </is>
+      </c>
+      <c r="E7" s="35" t="inlineStr"/>
+      <c r="F7" s="35" t="inlineStr"/>
+      <c r="G7" s="35" t="inlineStr"/>
+      <c r="H7" s="35" t="inlineStr"/>
+      <c r="I7" s="35" t="inlineStr"/>
+      <c r="J7" s="35" t="inlineStr"/>
+      <c r="K7" s="35" t="inlineStr"/>
+      <c r="L7" s="35" t="inlineStr"/>
+      <c r="M7" s="35" t="inlineStr"/>
+      <c r="N7" s="35" t="inlineStr"/>
+      <c r="O7" s="35" t="inlineStr"/>
+      <c r="P7" s="35" t="inlineStr"/>
+      <c r="Q7" s="35" t="inlineStr"/>
+      <c r="R7" s="35" t="inlineStr"/>
+      <c r="S7" s="35" t="inlineStr"/>
+      <c r="T7" s="35" t="inlineStr"/>
+      <c r="U7" s="35" t="inlineStr"/>
+      <c r="V7" s="35" t="inlineStr"/>
+      <c r="W7" s="35" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="X7" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y7" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z7" s="35" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="AA7" s="37" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="AB7" s="37" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AC7" s="35" t="inlineStr">
+        <is>
+          <t>stable</t>
+        </is>
+      </c>
+      <c r="AD7" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE7" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF7" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="AG7" s="35" t="inlineStr"/>
+      <c r="AH7" s="35" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" style="17" min="1" max="1"/>
+    <col width="40" customWidth="1" style="17" min="2" max="2"/>
+    <col width="120" customWidth="1" style="17" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="31" t="inlineStr">
+        <is>
+          <t>record_id</t>
+        </is>
+      </c>
+      <c r="B1" s="31" t="inlineStr">
+        <is>
+          <t>usage_json</t>
+        </is>
+      </c>
+      <c r="C1" s="31" t="inlineStr">
+        <is>
+          <t>raw_answers_json</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="35" t="inlineStr">
+        <is>
+          <t>R001</t>
+        </is>
+      </c>
+      <c r="B2" s="35" t="inlineStr">
+        <is>
+          <t>{"input_tokens": 465, "output_tokens": 92}</t>
+        </is>
+      </c>
+      <c r="C2" s="35" t="inlineStr">
+        <is>
+          <t>{"pump_failure_mode": {"type": "choice", "choice": "seal", "confidence": 1.0, "probabilities": {"cavitation": 0.0, "bearing": 0.0, "instrument": 0.0, "seal": 1.0, "other": 0.0}}, "pump_containment": {"type": "noul", "noul": 0.9}, "pump_urgency": {"type": "score", "score": 1.99, "confidence": 0.99, "legend": {"0": "Can wait for the next planned window", "1": "Should be handled within days", "2": "Needs attention now"}, "probabilities": {"0": 0.0, "1": 0.01, "2": 0.99}}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="35" t="inlineStr">
+        <is>
+          <t>R002</t>
+        </is>
+      </c>
+      <c r="B3" s="35" t="inlineStr">
+        <is>
+          <t>{"input_tokens": 464, "output_tokens": 92}</t>
+        </is>
+      </c>
+      <c r="C3" s="35" t="inlineStr">
+        <is>
+          <t>{"pump_failure_mode": {"type": "choice", "choice": "bearing", "confidence": 1.0, "probabilities": {"instrument": 0.0, "other": 0.0, "cavitation": 0.0, "seal": 0.0, "bearing": 1.0}}, "pump_containment": {"type": "noul", "noul": 0.01}, "pump_urgency": {"type": "score", "score": 0.01, "confidence": 0.99, "legend": {"0": "Can wait for the next planned window", "1": "Should be handled within days", "2": "Needs attention now"}, "probabilities": {"0": 0.99, "1": 0.01, "2": 0.0}}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="35" t="inlineStr">
+        <is>
+          <t>R003</t>
+        </is>
+      </c>
+      <c r="B4" s="35" t="inlineStr">
+        <is>
+          <t>{"input_tokens": 484, "output_tokens": 102}</t>
+        </is>
+      </c>
+      <c r="C4" s="35" t="inlineStr">
+        <is>
+          <t>{"hx_problem": {"type": "choice", "choice": "fouling", "confidence": 1.0, "probabilities": {"tube_leak": 0.0, "other": 0.0, "flow_maldistribution": 0.0, "control_valve": 0.0, "fouling": 1.0}}, "hx_crosscontam": {"type": "noul", "noul": 0.13}, "hx_impact": {"type": "score", "score": 1.09, "confidence": 0.86, "legend": {"0": "No noticeable impact", "1": "Reduced duty but operating", "2": "Major loss of duty or unit unusable"}, "probabilities": {"0": 0.0, "1": 0.91, "2": 0.09}}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="35" t="inlineStr">
+        <is>
+          <t>R004</t>
+        </is>
+      </c>
+      <c r="B5" s="35" t="inlineStr">
+        <is>
+          <t>{"input_tokens": 487, "output_tokens": 102}</t>
+        </is>
+      </c>
+      <c r="C5" s="35" t="inlineStr">
+        <is>
+          <t>{"hx_problem": {"type": "choice", "choice": "tube_leak", "confidence": 1.0, "probabilities": {"other": 0.0, "fouling": 0.0, "flow_maldistribution": 0.0, "tube_leak": 1.0, "control_valve": 0.0}}, "hx_crosscontam": {"type": "noul", "noul": 0.9}, "hx_impact": {"type": "score", "score": 1.27, "confidence": 0.49, "legend": {"0": "No noticeable impact", "1": "Reduced duty but operating", "2": "Major loss of duty or unit unusable"}, "probabilities": {"0": 0.04, "1": 0.66, "2": 0.3}}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="35" t="inlineStr">
+        <is>
+          <t>R005</t>
+        </is>
+      </c>
+      <c r="B6" s="35" t="inlineStr">
+        <is>
+          <t>{"input_tokens": 514, "output_tokens": 117}</t>
+        </is>
+      </c>
+      <c r="C6" s="35" t="inlineStr">
+        <is>
+          <t>{"col_symptom": {"type": "choice", "choice": "flooding", "confidence": 0.81, "probabilities": {"flooding": 0.84, "foaming": 0.08, "fouling": 0.01, "weeping": 0.0, "instrument": 0.04, "other": 0.03, "reboiler_condenser": 0.0}}, "col_offspec": {"type": "noul", "noul": 0.99}, "col_stability": {"type": "score", "score": 2.0, "confidence": 1.0, "legend": {"0": "Steady operation", "1": "Drifting or minor swings", "2": "Significant upset"}, "probabilities": {"0": 0.0, "1": 0.0, "2": 1.0}}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="35" t="inlineStr">
+        <is>
+          <t>R006</t>
+        </is>
+      </c>
+      <c r="B7" s="35" t="inlineStr">
+        <is>
+          <t>{"input_tokens": 512, "output_tokens": 115}</t>
+        </is>
+      </c>
+      <c r="C7" s="35" t="inlineStr">
+        <is>
+          <t>{"col_symptom": {"type": "choice", "choice": "other", "confidence": 1.0, "probabilities": {"weeping": 0.0, "instrument": 0.0, "foaming": 0.0, "flooding": 0.0, "reboiler_condenser": 0.0, "fouling": 0.0, "other": 1.0}}, "col_offspec": {"type": "noul", "noul": 0.01}, "col_stability": {"type": "score", "score": 0.0, "confidence": 1.0, "legend": {"0": "Steady operation", "1": "Drifting or minor swings", "2": "Significant upset"}, "probabilities": {"0": 1.0, "1": 0.0, "2": 0.0}}}</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" style="17" min="1" max="1"/>
+    <col width="10" customWidth="1" style="17" min="2" max="2"/>
+    <col width="8" customWidth="1" style="17" min="3" max="3"/>
+    <col width="10" customWidth="1" style="17" min="4" max="4"/>
+    <col width="18" customWidth="1" style="17" min="5" max="5"/>
+    <col width="16" customWidth="1" style="17" min="6" max="6"/>
+    <col width="14" customWidth="1" style="17" min="7" max="7"/>
+    <col width="9" customWidth="1" style="17" min="8" max="8"/>
+    <col width="10" customWidth="1" style="17" min="9" max="9"/>
+    <col width="20" customWidth="1" style="17" min="10" max="10"/>
+    <col width="20" customWidth="1" style="17" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="31" t="inlineStr">
+        <is>
+          <t>question_id</t>
+        </is>
+      </c>
+      <c r="B1" s="31" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="C1" s="31" t="inlineStr">
+        <is>
+          <t>asked</t>
+        </is>
+      </c>
+      <c r="D1" s="31" t="inlineStr">
+        <is>
+          <t>answered</t>
+        </is>
+      </c>
+      <c r="E1" s="31" t="inlineStr">
+        <is>
+          <t>flagged_for_review</t>
+        </is>
+      </c>
+      <c r="F1" s="31" t="inlineStr">
+        <is>
+          <t>mean_confidence</t>
+        </is>
+      </c>
+      <c r="G1" s="31" t="inlineStr">
+        <is>
+          <t>with_expected</t>
+        </is>
+      </c>
+      <c r="H1" s="31" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
+      <c r="I1" s="31" t="inlineStr">
+        <is>
+          <t>accuracy</t>
+        </is>
+      </c>
+      <c r="J1" s="31" t="inlineStr">
+        <is>
+          <t>mean_conf_when_correct</t>
+        </is>
+      </c>
+      <c r="K1" s="31" t="inlineStr">
+        <is>
+          <t>mean_conf_when_wrong</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="35" t="inlineStr">
+        <is>
+          <t>pump_failure_mode</t>
+        </is>
+      </c>
+      <c r="B2" s="35" t="inlineStr">
+        <is>
+          <t>choice</t>
+        </is>
+      </c>
+      <c r="C2" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="H2" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="I2" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" s="35" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="35" t="inlineStr">
+        <is>
+          <t>pump_containment</t>
+        </is>
+      </c>
+      <c r="B3" s="35" t="inlineStr">
+        <is>
+          <t>noul</t>
+        </is>
+      </c>
+      <c r="C3" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="35" t="n">
+        <v>0.945</v>
+      </c>
+      <c r="G3" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="I3" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" s="35" t="n">
+        <v>0.945</v>
+      </c>
+      <c r="K3" s="35" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="35" t="inlineStr">
+        <is>
+          <t>pump_urgency</t>
+        </is>
+      </c>
+      <c r="B4" s="35" t="inlineStr">
+        <is>
+          <t>score</t>
+        </is>
+      </c>
+      <c r="C4" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="35" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G4" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="H4" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="I4" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" s="35" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="K4" s="35" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="35" t="inlineStr">
+        <is>
+          <t>hx_problem</t>
+        </is>
+      </c>
+      <c r="B5" s="35" t="inlineStr">
+        <is>
+          <t>choice</t>
+        </is>
+      </c>
+      <c r="C5" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="H5" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="I5" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" s="35" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="35" t="inlineStr">
+        <is>
+          <t>hx_crosscontam</t>
+        </is>
+      </c>
+      <c r="B6" s="35" t="inlineStr">
+        <is>
+          <t>noul</t>
+        </is>
+      </c>
+      <c r="C6" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="35" t="n">
+        <v>0.885</v>
+      </c>
+      <c r="G6" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="35" t="n">
+        <v>0.885</v>
+      </c>
+      <c r="K6" s="35" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="35" t="inlineStr">
+        <is>
+          <t>hx_impact</t>
+        </is>
+      </c>
+      <c r="B7" s="35" t="inlineStr">
+        <is>
+          <t>score</t>
+        </is>
+      </c>
+      <c r="C7" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="35" t="n">
+        <v>0.675</v>
+      </c>
+      <c r="G7" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="35" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J7" s="35" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="K7" s="35" t="n">
+        <v>0.49</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="35" t="inlineStr">
+        <is>
+          <t>col_symptom</t>
+        </is>
+      </c>
+      <c r="B8" s="35" t="inlineStr">
+        <is>
+          <t>choice</t>
+        </is>
+      </c>
+      <c r="C8" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="35" t="n">
+        <v>0.905</v>
+      </c>
+      <c r="G8" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="I8" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" s="35" t="n">
+        <v>0.905</v>
+      </c>
+      <c r="K8" s="35" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="35" t="inlineStr">
+        <is>
+          <t>col_offspec</t>
+        </is>
+      </c>
+      <c r="B9" s="35" t="inlineStr">
+        <is>
+          <t>noul</t>
+        </is>
+      </c>
+      <c r="C9" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="35" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G9" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="H9" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="I9" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" s="35" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="K9" s="35" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="35" t="inlineStr">
+        <is>
+          <t>col_stability</t>
+        </is>
+      </c>
+      <c r="B10" s="35" t="inlineStr">
+        <is>
+          <t>score</t>
+        </is>
+      </c>
+      <c r="C10" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="I10" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="35" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" style="17" min="1" max="1"/>
+    <col width="70" customWidth="1" style="17" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="31" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="B1" s="31" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="35" t="inlineStr">
+        <is>
+          <t>run_started</t>
+        </is>
+      </c>
+      <c r="B2" s="35" t="inlineStr">
+        <is>
+          <t>20260930_142230</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="35" t="inlineStr">
+        <is>
+          <t>workbook</t>
+        </is>
+      </c>
+      <c r="B3" s="35" t="inlineStr">
+        <is>
+          <t>/mnt/d/dev/nimble_plant/nimble_classifier_workbook.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="35" t="inlineStr">
+        <is>
+          <t>engine</t>
+        </is>
+      </c>
+      <c r="B4" s="35" t="inlineStr">
+        <is>
+          <t>jev</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="35" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="B5" s="35" t="inlineStr">
+        <is>
+          <t>jev-1.13.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="35" t="inlineStr">
+        <is>
+          <t>base_url</t>
+        </is>
+      </c>
+      <c r="B6" s="35" t="inlineStr">
+        <is>
+          <t>https://api.typesafe.ai</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="35" t="inlineStr">
+        <is>
+          <t>endpoint_info</t>
+        </is>
+      </c>
+      <c r="B7" s="35" t="inlineStr">
+        <is>
+          <t>remote:https://api.typesafe.ai</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="35" t="inlineStr">
+        <is>
+          <t>questions_hash</t>
+        </is>
+      </c>
+      <c r="B8" s="35" t="inlineStr">
+        <is>
+          <t>f73a405167a3</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="35" t="inlineStr">
+        <is>
+          <t>api_key_configured</t>
+        </is>
+      </c>
+      <c r="B9" s="35" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="35" t="inlineStr">
+        <is>
+          <t>records_in_run</t>
+        </is>
+      </c>
+      <c r="B10" s="35" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="35" t="inlineStr">
+        <is>
+          <t>records_completed</t>
+        </is>
+      </c>
+      <c r="B11" s="35" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="35" t="inlineStr">
+        <is>
+          <t>failed_records</t>
+        </is>
+      </c>
+      <c r="B12" s="35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="35" t="inlineStr">
+        <is>
+          <t>review_threshold_default</t>
+        </is>
+      </c>
       <c r="B13" s="35" t="inlineStr">
         <is>
-          <t>output_Results, output_Raw, output_Summary, output_Run_info</t>
-        </is>
+          <t>0.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="35" t="inlineStr">
+        <is>
+          <t>elapsed_seconds</t>
+        </is>
+      </c>
+      <c r="B14" s="35" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="35" t="inlineStr">
+        <is>
+          <t>checkpoint</t>
+        </is>
+      </c>
+      <c r="B15" s="35" t="inlineStr">
+        <is>
+          <t>/mnt/d/dev/nimble_plant/nimble_classifier_workbook_jev_20260930_142230.jsonl</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="35" t="inlineStr">
+        <is>
+          <t>input_tokens</t>
+        </is>
+      </c>
+      <c r="B16" s="35" t="inlineStr">
+        <is>
+          <t>2926</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="35" t="inlineStr">
+        <is>
+          <t>output_tokens</t>
+        </is>
+      </c>
+      <c r="B17" s="35" t="inlineStr">
+        <is>
+          <t>620</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="35" t="inlineStr">
+        <is>
+          <t>total_tokens</t>
+        </is>
+      </c>
+      <c r="B18" s="35" t="inlineStr">
+        <is>
+          <t>3546</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="35" t="inlineStr">
+        <is>
+          <t>records_with_usage</t>
+        </is>
+      </c>
+      <c r="B19" s="35" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="35" t="inlineStr">
+        <is>
+          <t>output_sheets</t>
+        </is>
+      </c>
+      <c r="B20" s="35" t="inlineStr">
+        <is>
+          <t>output_jev_Results, output_jev_Raw, output_jev_Summary, output_jev_Run_info</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" style="17" min="1" max="1"/>
+    <col width="22" customWidth="1" style="17" min="2" max="2"/>
+    <col width="14" customWidth="1" style="17" min="3" max="3"/>
+    <col width="14" customWidth="1" style="17" min="4" max="4"/>
+    <col width="8" customWidth="1" style="17" min="5" max="5"/>
+    <col width="14" customWidth="1" style="17" min="6" max="6"/>
+    <col width="14" customWidth="1" style="17" min="7" max="7"/>
+    <col width="12" customWidth="1" style="17" min="8" max="8"/>
+    <col width="12" customWidth="1" style="17" min="9" max="9"/>
+    <col width="12" customWidth="1" style="17" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="31" t="inlineStr">
+        <is>
+          <t>record_id</t>
+        </is>
+      </c>
+      <c r="B1" s="31" t="inlineStr">
+        <is>
+          <t>question_id</t>
+        </is>
+      </c>
+      <c r="C1" s="31" t="inlineStr">
+        <is>
+          <t>nimble_answer</t>
+        </is>
+      </c>
+      <c r="D1" s="31" t="inlineStr">
+        <is>
+          <t>jev_answer</t>
+        </is>
+      </c>
+      <c r="E1" s="31" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="F1" s="31" t="inlineStr">
+        <is>
+          <t>nimble_confidence</t>
+        </is>
+      </c>
+      <c r="G1" s="31" t="inlineStr">
+        <is>
+          <t>jev_confidence</t>
+        </is>
+      </c>
+      <c r="H1" s="31" t="inlineStr">
+        <is>
+          <t>expected</t>
+        </is>
+      </c>
+      <c r="I1" s="31" t="inlineStr">
+        <is>
+          <t>nimble_correct</t>
+        </is>
+      </c>
+      <c r="J1" s="31" t="inlineStr">
+        <is>
+          <t>jev_correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="35" t="inlineStr">
+        <is>
+          <t>R001</t>
+        </is>
+      </c>
+      <c r="B2" s="35" t="inlineStr">
+        <is>
+          <t>pump_containment</t>
+        </is>
+      </c>
+      <c r="C2" s="35" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="D2" s="35" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E2" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="F2" s="35" t="n">
+        <v>0.9347743692709441</v>
+      </c>
+      <c r="G2" s="35" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H2" s="35" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I2" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="J2" s="35" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="35" t="inlineStr">
+        <is>
+          <t>R001</t>
+        </is>
+      </c>
+      <c r="B3" s="35" t="inlineStr">
+        <is>
+          <t>pump_failure_mode</t>
+        </is>
+      </c>
+      <c r="C3" s="35" t="inlineStr">
+        <is>
+          <t>seal</t>
+        </is>
+      </c>
+      <c r="D3" s="35" t="inlineStr">
+        <is>
+          <t>seal</t>
+        </is>
+      </c>
+      <c r="E3" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="F3" s="35" t="n">
+        <v>0.886096743401824</v>
+      </c>
+      <c r="G3" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" s="35" t="inlineStr">
+        <is>
+          <t>seal</t>
+        </is>
+      </c>
+      <c r="I3" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="J3" s="35" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="35" t="inlineStr">
+        <is>
+          <t>R001</t>
+        </is>
+      </c>
+      <c r="B4" s="35" t="inlineStr">
+        <is>
+          <t>pump_urgency</t>
+        </is>
+      </c>
+      <c r="C4" s="35" t="inlineStr">
+        <is>
+          <t>immediate</t>
+        </is>
+      </c>
+      <c r="D4" s="35" t="inlineStr">
+        <is>
+          <t>immediate</t>
+        </is>
+      </c>
+      <c r="E4" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="F4" s="35" t="n">
+        <v>0.5139963542213443</v>
+      </c>
+      <c r="G4" s="35" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H4" s="35" t="inlineStr">
+        <is>
+          <t>immediate</t>
+        </is>
+      </c>
+      <c r="I4" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="J4" s="35" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="35" t="inlineStr">
+        <is>
+          <t>R002</t>
+        </is>
+      </c>
+      <c r="B5" s="35" t="inlineStr">
+        <is>
+          <t>pump_containment</t>
+        </is>
+      </c>
+      <c r="C5" s="35" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D5" s="35" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E5" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="F5" s="35" t="n">
+        <v>0.9908501157291482</v>
+      </c>
+      <c r="G5" s="35" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H5" s="35" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="I5" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="J5" s="35" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="35" t="inlineStr">
+        <is>
+          <t>R002</t>
+        </is>
+      </c>
+      <c r="B6" s="35" t="inlineStr">
+        <is>
+          <t>pump_failure_mode</t>
+        </is>
+      </c>
+      <c r="C6" s="35" t="inlineStr">
+        <is>
+          <t>bearing</t>
+        </is>
+      </c>
+      <c r="D6" s="35" t="inlineStr">
+        <is>
+          <t>bearing</t>
+        </is>
+      </c>
+      <c r="E6" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="F6" s="35" t="n">
+        <v>0.971844626140937</v>
+      </c>
+      <c r="G6" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="35" t="inlineStr">
+        <is>
+          <t>bearing</t>
+        </is>
+      </c>
+      <c r="I6" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="J6" s="35" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="35" t="inlineStr">
+        <is>
+          <t>R002</t>
+        </is>
+      </c>
+      <c r="B7" s="35" t="inlineStr">
+        <is>
+          <t>pump_urgency</t>
+        </is>
+      </c>
+      <c r="C7" s="35" t="inlineStr">
+        <is>
+          <t>routine</t>
+        </is>
+      </c>
+      <c r="D7" s="35" t="inlineStr">
+        <is>
+          <t>routine</t>
+        </is>
+      </c>
+      <c r="E7" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="F7" s="35" t="n">
+        <v>0.942439470709464</v>
+      </c>
+      <c r="G7" s="35" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H7" s="35" t="inlineStr">
+        <is>
+          <t>routine</t>
+        </is>
+      </c>
+      <c r="I7" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="J7" s="35" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="35" t="inlineStr">
+        <is>
+          <t>R003</t>
+        </is>
+      </c>
+      <c r="B8" s="35" t="inlineStr">
+        <is>
+          <t>hx_crosscontam</t>
+        </is>
+      </c>
+      <c r="C8" s="35" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D8" s="35" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E8" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="F8" s="35" t="n">
+        <v>0.9778307138401591</v>
+      </c>
+      <c r="G8" s="35" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="H8" s="35" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="I8" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="J8" s="35" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="35" t="inlineStr">
+        <is>
+          <t>R003</t>
+        </is>
+      </c>
+      <c r="B9" s="35" t="inlineStr">
+        <is>
+          <t>hx_impact</t>
+        </is>
+      </c>
+      <c r="C9" s="35" t="inlineStr">
+        <is>
+          <t>degraded</t>
+        </is>
+      </c>
+      <c r="D9" s="35" t="inlineStr">
+        <is>
+          <t>degraded</t>
+        </is>
+      </c>
+      <c r="E9" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="F9" s="35" t="n">
+        <v>0.1302623881325073</v>
+      </c>
+      <c r="G9" s="35" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="H9" s="35" t="inlineStr">
+        <is>
+          <t>degraded</t>
+        </is>
+      </c>
+      <c r="I9" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="J9" s="35" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="35" t="inlineStr">
+        <is>
+          <t>R003</t>
+        </is>
+      </c>
+      <c r="B10" s="35" t="inlineStr">
+        <is>
+          <t>hx_problem</t>
+        </is>
+      </c>
+      <c r="C10" s="35" t="inlineStr">
+        <is>
+          <t>fouling</t>
+        </is>
+      </c>
+      <c r="D10" s="35" t="inlineStr">
+        <is>
+          <t>fouling</t>
+        </is>
+      </c>
+      <c r="E10" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="F10" s="35" t="n">
+        <v>0.8436129076949702</v>
+      </c>
+      <c r="G10" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="35" t="inlineStr">
+        <is>
+          <t>fouling</t>
+        </is>
+      </c>
+      <c r="I10" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="J10" s="35" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="35" t="inlineStr">
+        <is>
+          <t>R004</t>
+        </is>
+      </c>
+      <c r="B11" s="35" t="inlineStr">
+        <is>
+          <t>hx_crosscontam</t>
+        </is>
+      </c>
+      <c r="C11" s="35" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="D11" s="35" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E11" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="F11" s="35" t="n">
+        <v>0.9973633152102099</v>
+      </c>
+      <c r="G11" s="35" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H11" s="35" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I11" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="J11" s="35" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="35" t="inlineStr">
+        <is>
+          <t>R004</t>
+        </is>
+      </c>
+      <c r="B12" s="35" t="inlineStr">
+        <is>
+          <t>hx_impact</t>
+        </is>
+      </c>
+      <c r="C12" s="35" t="inlineStr">
+        <is>
+          <t>degraded</t>
+        </is>
+      </c>
+      <c r="D12" s="35" t="inlineStr">
+        <is>
+          <t>degraded</t>
+        </is>
+      </c>
+      <c r="E12" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="F12" s="35" t="n">
+        <v>0.5160678099489566</v>
+      </c>
+      <c r="G12" s="35" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="H12" s="35" t="inlineStr">
+        <is>
+          <t>severe</t>
+        </is>
+      </c>
+      <c r="I12" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="J12" s="35" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="35" t="inlineStr">
+        <is>
+          <t>R004</t>
+        </is>
+      </c>
+      <c r="B13" s="35" t="inlineStr">
+        <is>
+          <t>hx_problem</t>
+        </is>
+      </c>
+      <c r="C13" s="35" t="inlineStr">
+        <is>
+          <t>tube_leak</t>
+        </is>
+      </c>
+      <c r="D13" s="35" t="inlineStr">
+        <is>
+          <t>tube_leak</t>
+        </is>
+      </c>
+      <c r="E13" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="F13" s="35" t="n">
+        <v>0.9809344898041918</v>
+      </c>
+      <c r="G13" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" s="35" t="inlineStr">
+        <is>
+          <t>tube_leak</t>
+        </is>
+      </c>
+      <c r="I13" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="J13" s="35" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="35" t="inlineStr">
+        <is>
+          <t>R005</t>
+        </is>
+      </c>
+      <c r="B14" s="35" t="inlineStr">
+        <is>
+          <t>col_offspec</t>
+        </is>
+      </c>
+      <c r="C14" s="35" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="D14" s="35" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E14" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="F14" s="35" t="n">
+        <v>0.9990587441403763</v>
+      </c>
+      <c r="G14" s="35" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H14" s="35" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I14" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="J14" s="35" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="35" t="inlineStr">
+        <is>
+          <t>R005</t>
+        </is>
+      </c>
+      <c r="B15" s="35" t="inlineStr">
+        <is>
+          <t>col_stability</t>
+        </is>
+      </c>
+      <c r="C15" s="35" t="inlineStr">
+        <is>
+          <t>upset</t>
+        </is>
+      </c>
+      <c r="D15" s="35" t="inlineStr">
+        <is>
+          <t>upset</t>
+        </is>
+      </c>
+      <c r="E15" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="F15" s="35" t="n">
+        <v>0.6363997745790606</v>
+      </c>
+      <c r="G15" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="35" t="inlineStr">
+        <is>
+          <t>upset</t>
+        </is>
+      </c>
+      <c r="I15" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="J15" s="35" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="35" t="inlineStr">
+        <is>
+          <t>R005</t>
+        </is>
+      </c>
+      <c r="B16" s="35" t="inlineStr">
+        <is>
+          <t>col_symptom</t>
+        </is>
+      </c>
+      <c r="C16" s="35" t="inlineStr">
+        <is>
+          <t>flooding</t>
+        </is>
+      </c>
+      <c r="D16" s="35" t="inlineStr">
+        <is>
+          <t>flooding</t>
+        </is>
+      </c>
+      <c r="E16" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="F16" s="35" t="n">
+        <v>0.5761713560101278</v>
+      </c>
+      <c r="G16" s="35" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="H16" s="35" t="inlineStr">
+        <is>
+          <t>flooding</t>
+        </is>
+      </c>
+      <c r="I16" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="J16" s="35" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="35" t="inlineStr">
+        <is>
+          <t>R006</t>
+        </is>
+      </c>
+      <c r="B17" s="35" t="inlineStr">
+        <is>
+          <t>col_offspec</t>
+        </is>
+      </c>
+      <c r="C17" s="35" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D17" s="35" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E17" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="F17" s="35" t="n">
+        <v>0.9979530469785511</v>
+      </c>
+      <c r="G17" s="35" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H17" s="35" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="I17" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="J17" s="35" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="35" t="inlineStr">
+        <is>
+          <t>R006</t>
+        </is>
+      </c>
+      <c r="B18" s="35" t="inlineStr">
+        <is>
+          <t>col_stability</t>
+        </is>
+      </c>
+      <c r="C18" s="35" t="inlineStr">
+        <is>
+          <t>stable</t>
+        </is>
+      </c>
+      <c r="D18" s="35" t="inlineStr">
+        <is>
+          <t>stable</t>
+        </is>
+      </c>
+      <c r="E18" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="F18" s="35" t="n">
+        <v>0.980965088363793</v>
+      </c>
+      <c r="G18" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="35" t="inlineStr">
+        <is>
+          <t>stable</t>
+        </is>
+      </c>
+      <c r="I18" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="J18" s="35" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="35" t="inlineStr">
+        <is>
+          <t>R006</t>
+        </is>
+      </c>
+      <c r="B19" s="35" t="inlineStr">
+        <is>
+          <t>col_symptom</t>
+        </is>
+      </c>
+      <c r="C19" s="35" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="D19" s="35" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="E19" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="F19" s="35" t="n">
+        <v>0.9310185171064398</v>
+      </c>
+      <c r="G19" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="35" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="I19" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="J19" s="35" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1067,173 +3494,203 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="26" customWidth="1" style="16" min="1" max="1"/>
-    <col width="34" customWidth="1" style="16" min="2" max="2"/>
-    <col width="80" customWidth="1" style="16" min="3" max="3"/>
+    <col width="22" customWidth="1" style="16" min="1" max="1"/>
+    <col width="28" customWidth="1" style="16" min="2" max="2"/>
+    <col width="90" customWidth="1" style="16" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="17">
-      <c r="A1" s="25" t="inlineStr">
+      <c r="A1" s="47" t="inlineStr">
         <is>
           <t>key</t>
         </is>
       </c>
-      <c r="B1" s="25" t="inlineStr">
+      <c r="B1" s="47" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
-      <c r="C1" s="25" t="inlineStr">
+      <c r="C1" s="47" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="17">
-      <c r="A2" s="26" t="inlineStr">
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>engine</t>
+        </is>
+      </c>
+      <c r="B2" s="16" t="inlineStr">
+        <is>
+          <t>nimble</t>
+        </is>
+      </c>
+      <c r="C2" s="16" t="inlineStr">
+        <is>
+          <t>nimble (local Ollama) or jev (TypeSafe). CLI --engine overrides this. Preset sets model/base_url/endpoint.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1" s="17">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="B2" s="27" t="inlineStr">
+      <c r="B3" s="16" t="inlineStr">
         <is>
           <t>nimble</t>
         </is>
       </c>
-      <c r="C2" s="28" t="inlineStr">
-        <is>
-          <t>Ollama model name. Must be pulled first (ollama pull nimble). Requires Ollama 0.35 or later.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="17">
-      <c r="A3" s="26" t="inlineStr">
+      <c r="C3" s="16" t="inlineStr">
+        <is>
+          <t>Overridden by engine preset at runtime (nimble or jev-1.13.0). Kept for reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="17">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>base_url</t>
         </is>
       </c>
-      <c r="B3" s="27" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr">
         <is>
           <t>http://localhost:11434</t>
         </is>
       </c>
-      <c r="C3" s="28" t="inlineStr">
-        <is>
-          <t>Ollama server address.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="17">
-      <c r="A4" s="26" t="inlineStr">
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>Overridden by engine preset (localhost:11434 or https://api.typesafe.ai).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1" s="17">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>endpoint</t>
         </is>
       </c>
-      <c r="B4" s="27" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>/v1/systemone</t>
         </is>
       </c>
-      <c r="C4" s="28" t="inlineStr">
-        <is>
-          <t>Decision-model endpoint.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="15" customHeight="1" s="17">
-      <c r="A5" s="26" t="inlineStr">
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Decision-model endpoint (same for both engines).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1" s="17">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>timeout_seconds</t>
         </is>
       </c>
-      <c r="B5" s="27" t="n">
+      <c r="B6" s="16" t="n">
         <v>120</v>
       </c>
-      <c r="C5" s="28" t="inlineStr">
+      <c r="C6" s="16" t="inlineStr">
         <is>
           <t>Per-request timeout.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" s="17">
-      <c r="A6" s="26" t="inlineStr">
+    <row r="7" ht="23.85" customHeight="1" s="17">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>retries</t>
         </is>
       </c>
-      <c r="B6" s="27" t="n">
+      <c r="B7" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="C6" s="28" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
         <is>
           <t>Retries per record after a failed request.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="23.85" customHeight="1" s="17">
-      <c r="A7" s="26" t="inlineStr">
+    <row r="8" ht="15" customHeight="1" s="17">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>default_review_below</t>
         </is>
       </c>
-      <c r="B7" s="27" t="n">
+      <c r="B8" s="16" t="n">
         <v>0.6</v>
       </c>
-      <c r="C7" s="28" t="inlineStr">
+      <c r="C8" s="16" t="inlineStr">
         <is>
           <t>Placeholder threshold. Rows with confidence below this are flagged for review. Tune on records with known answers.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" s="17">
-      <c r="A8" s="26" t="inlineStr">
+    <row r="9" ht="15" customHeight="1" s="17">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>test_first_n</t>
         </is>
       </c>
-      <c r="B8" s="27" t="n">
+      <c r="B9" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="C8" s="28" t="inlineStr">
+      <c r="C9" s="16" t="inlineStr">
         <is>
           <t>Number of records processed in test mode. Set to blank or 0 to disable.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" s="17">
-      <c r="A9" s="26" t="inlineStr">
+    <row r="10" ht="15" customHeight="1" s="17">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>record_text_column</t>
         </is>
       </c>
-      <c r="B9" s="27" t="inlineStr">
+      <c r="B10" s="16" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="C9" s="28" t="inlineStr">
+      <c r="C10" s="16" t="inlineStr">
         <is>
           <t>Name of the Records column that holds the statement.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1" s="17">
-      <c r="A10" s="26" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>output_prefix</t>
         </is>
       </c>
-      <c r="B10" s="27" t="inlineStr">
+      <c r="B11" s="16" t="inlineStr">
         <is>
           <t>nimble_results</t>
         </is>
       </c>
-      <c r="C10" s="28" t="inlineStr">
-        <is>
-          <t>Legacy. Checkpoints are named &lt;workbook_stem&gt;_&lt;timestamp&gt;.jsonl beside the workbook. Excel results use output_* sheets.</t>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Legacy. Results use output_&lt;engine&gt;_* sheets; checkpoints are &lt;workbook&gt;_&lt;engine&gt;_&lt;timestamp&gt;.jsonl.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>api_key</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="inlineStr"/>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>Leave blank. Prefer export TYPESAFE_API_KEY=... for Jev (never commit a key).</t>
         </is>
       </c>
     </row>
@@ -16014,10 +18471,10 @@
         </is>
       </c>
       <c r="F2" s="34" t="n">
-        <v>0.8845493270621723</v>
+        <v>0.886096743401824</v>
       </c>
       <c r="G2" s="34" t="n">
-        <v>0.9656847333764127</v>
+        <v>0.9662224910900805</v>
       </c>
       <c r="H2" s="32" t="inlineStr">
         <is>
@@ -16025,10 +18482,10 @@
         </is>
       </c>
       <c r="I2" s="34" t="n">
-        <v>0.9344222768578154</v>
+        <v>0.9347743692709441</v>
       </c>
       <c r="J2" s="34" t="n">
-        <v>0.9344222768578154</v>
+        <v>0.9347743692709441</v>
       </c>
       <c r="K2" s="32" t="inlineStr">
         <is>
@@ -16036,10 +18493,10 @@
         </is>
       </c>
       <c r="L2" s="34" t="n">
-        <v>0.5092630137668384</v>
+        <v>0.5139963542213443</v>
       </c>
       <c r="M2" s="34" t="n">
-        <v>1.792500181836202</v>
+        <v>1.795605456964634</v>
       </c>
       <c r="N2" s="32" t="inlineStr"/>
       <c r="O2" s="32" t="inlineStr"/>
@@ -16096,10 +18553,10 @@
         </is>
       </c>
       <c r="F3" s="37" t="n">
-        <v>0.9714843129418362</v>
+        <v>0.971844626140937</v>
       </c>
       <c r="G3" s="37" t="n">
-        <v>0.9934575546721711</v>
+        <v>0.9935691479963884</v>
       </c>
       <c r="H3" s="35" t="inlineStr">
         <is>
@@ -16107,10 +18564,10 @@
         </is>
       </c>
       <c r="I3" s="37" t="n">
-        <v>0.9911026645183536</v>
+        <v>0.9908501157291482</v>
       </c>
       <c r="J3" s="37" t="n">
-        <v>0.008897335481646413</v>
+        <v>0.009149884270851874</v>
       </c>
       <c r="K3" s="35" t="inlineStr">
         <is>
@@ -16118,10 +18575,10 @@
         </is>
       </c>
       <c r="L3" s="37" t="n">
-        <v>0.9435743291549853</v>
+        <v>0.942439470709464</v>
       </c>
       <c r="M3" s="37" t="n">
-        <v>0.01215235614936457</v>
+        <v>0.01254440492998592</v>
       </c>
       <c r="N3" s="35" t="inlineStr"/>
       <c r="O3" s="35" t="inlineStr"/>
@@ -16183,10 +18640,10 @@
         </is>
       </c>
       <c r="O4" s="34" t="n">
-        <v>0.8435687329991992</v>
+        <v>0.8436129076949702</v>
       </c>
       <c r="P4" s="34" t="n">
-        <v>0.9478850419472986</v>
+        <v>0.9479736032978536</v>
       </c>
       <c r="Q4" s="32" t="inlineStr">
         <is>
@@ -16194,10 +18651,10 @@
         </is>
       </c>
       <c r="R4" s="34" t="n">
-        <v>0.9770510463918108</v>
+        <v>0.9778307138401591</v>
       </c>
       <c r="S4" s="34" t="n">
-        <v>0.02294895360818915</v>
+        <v>0.02216928615984095</v>
       </c>
       <c r="T4" s="32" t="inlineStr">
         <is>
@@ -16205,10 +18662,10 @@
         </is>
       </c>
       <c r="U4" s="34" t="n">
-        <v>0.1334007415612771</v>
+        <v>0.1302623881325073</v>
       </c>
       <c r="V4" s="34" t="n">
-        <v>1.315495834073972</v>
+        <v>1.300448838097414</v>
       </c>
       <c r="W4" s="32" t="inlineStr"/>
       <c r="X4" s="32" t="inlineStr"/>
@@ -16265,10 +18722,10 @@
         </is>
       </c>
       <c r="O5" s="34" t="n">
-        <v>0.9811052724756711</v>
+        <v>0.9809344898041918</v>
       </c>
       <c r="P5" s="34" t="n">
-        <v>0.9959796555651736</v>
+        <v>0.9959396543190018</v>
       </c>
       <c r="Q5" s="32" t="inlineStr">
         <is>
@@ -16276,10 +18733,10 @@
         </is>
       </c>
       <c r="R5" s="34" t="n">
-        <v>0.9972773611314817</v>
+        <v>0.9973633152102099</v>
       </c>
       <c r="S5" s="34" t="n">
-        <v>0.9972773611314817</v>
+        <v>0.9973633152102099</v>
       </c>
       <c r="T5" s="32" t="inlineStr">
         <is>
@@ -16287,10 +18744,10 @@
         </is>
       </c>
       <c r="U5" s="34" t="n">
-        <v>0.5167403657884981</v>
+        <v>0.5160678099489566</v>
       </c>
       <c r="V5" s="34" t="n">
-        <v>1.011186618395636</v>
+        <v>1.01263221363486</v>
       </c>
       <c r="W5" s="32" t="inlineStr"/>
       <c r="X5" s="32" t="inlineStr"/>
@@ -16356,10 +18813,10 @@
         </is>
       </c>
       <c r="X6" s="34" t="n">
-        <v>0.575229541784642</v>
+        <v>0.5761713560101278</v>
       </c>
       <c r="Y6" s="34" t="n">
-        <v>0.5175961061389851</v>
+        <v>0.5213366239870925</v>
       </c>
       <c r="Z6" s="32" t="inlineStr">
         <is>
@@ -16367,10 +18824,10 @@
         </is>
       </c>
       <c r="AA6" s="34" t="n">
-        <v>0.9990573225259095</v>
+        <v>0.9990587441403763</v>
       </c>
       <c r="AB6" s="34" t="n">
-        <v>0.9990573225259095</v>
+        <v>0.9990587441403763</v>
       </c>
       <c r="AC6" s="32" t="inlineStr">
         <is>
@@ -16378,10 +18835,10 @@
         </is>
       </c>
       <c r="AD6" s="34" t="n">
-        <v>0.6360617217354828</v>
+        <v>0.6363997745790606</v>
       </c>
       <c r="AE6" s="34" t="n">
-        <v>1.81944012506878</v>
+        <v>1.819090602596957</v>
       </c>
       <c r="AF6" s="32" t="b">
         <v>1</v>
@@ -16438,10 +18895,10 @@
         </is>
       </c>
       <c r="X7" s="37" t="n">
-        <v>0.9294495624188652</v>
+        <v>0.9310185171064398</v>
       </c>
       <c r="Y7" s="37" t="n">
-        <v>0.9729023573239992</v>
+        <v>0.9736380706169232</v>
       </c>
       <c r="Z7" s="35" t="inlineStr">
         <is>
@@ -16449,10 +18906,10 @@
         </is>
       </c>
       <c r="AA7" s="37" t="n">
-        <v>0.9980349345556877</v>
+        <v>0.9979530469785511</v>
       </c>
       <c r="AB7" s="37" t="n">
-        <v>0.001965065444312336</v>
+        <v>0.002046953021448908</v>
       </c>
       <c r="AC7" s="35" t="inlineStr">
         <is>
@@ -16460,10 +18917,10 @@
         </is>
       </c>
       <c r="AD7" s="37" t="n">
-        <v>0.9805633856279246</v>
+        <v>0.980965088363793</v>
       </c>
       <c r="AE7" s="37" t="n">
-        <v>0.004745121587660906</v>
+        <v>0.004613240175433055</v>
       </c>
       <c r="AF7" s="35" t="b">
         <v>0</v>
@@ -16482,11 +18939,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="17" min="1" max="1"/>
-    <col width="120" customWidth="1" style="17" min="2" max="2"/>
+    <col width="40" customWidth="1" style="17" min="2" max="2"/>
+    <col width="120" customWidth="1" style="17" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -16497,6 +18955,11 @@
       </c>
       <c r="B1" s="31" t="inlineStr">
         <is>
+          <t>usage_json</t>
+        </is>
+      </c>
+      <c r="C1" s="31" t="inlineStr">
+        <is>
           <t>raw_answers_json</t>
         </is>
       </c>
@@ -16509,7 +18972,12 @@
       </c>
       <c r="B2" s="35" t="inlineStr">
         <is>
-          <t>{"pump_failure_mode": {"type": "choice", "choice": "seal", "probabilities": {"seal": 0.9656847333764127, "bearing": 0.012815798358892808, "cavitation": 0.01719299268622746, "instrument": 0.0018161557694942427, "other": 0.0024903198089730396}, "confidence": 0.8845493270621723}, "pump_containment": {"type": "noul", "noul": 0.9344222768578154}, "pump_urgency": {"type": "score", "score": 1.7925001818362023, "legend": {"0": "Can wait for the next planned window", "1": "Should be handled within days", "2": "Needs attention now"}, "probabilities": {"0": 0.045530782702412724, "1": 0.11643825275897222, "2": 0.838030964538615}, "confidence": 0.5092630137668384}}</t>
+          <t>{"input_tokens": 1063, "output_tokens": 4}</t>
+        </is>
+      </c>
+      <c r="C2" s="35" t="inlineStr">
+        <is>
+          <t>{"pump_failure_mode": {"type": "choice", "choice": "seal", "probabilities": {"seal": 0.9662224910900805, "bearing": 0.012618353313619128, "cavitation": 0.01697751866187461, "instrument": 0.0017525858181681566, "other": 0.0024290511162574644}, "confidence": 0.886096743401824}, "pump_containment": {"type": "noul", "noul": 0.9347743692709441}, "pump_urgency": {"type": "score", "score": 1.7956054569646345, "legend": {"0": "Can wait for the next planned window", "1": "Should be handled within days", "2": "Needs attention now"}, "probabilities": {"0": 0.04461471259079198, "1": 0.11516511785378156, "2": 0.8402201695554264}, "confidence": 0.5139963542213443}}</t>
         </is>
       </c>
     </row>
@@ -16521,7 +18989,12 @@
       </c>
       <c r="B3" s="35" t="inlineStr">
         <is>
-          <t>{"pump_failure_mode": {"type": "choice", "choice": "bearing", "probabilities": {"seal": 0.0043512978021535585, "bearing": 0.9934575546721711, "cavitation": 0.000905819088747979, "instrument": 0.0004185861337592025, "other": 0.0008667423031681805}, "confidence": 0.9714843129418362}, "pump_containment": {"type": "noul", "noul": 0.008897335481646413}, "pump_urgency": {"type": "score", "score": 0.012152356149364569, "legend": {"0": "Can wait for the next planned window", "1": "Should be handled within days", "2": "Needs attention now"}, "probabilities": {"0": 0.9897726497601865, "1": 0.008302344330262468, "2": 0.0019250059095510502}, "confidence": 0.9435743291549853}}</t>
+          <t>{"input_tokens": 1066, "output_tokens": 4}</t>
+        </is>
+      </c>
+      <c r="C3" s="35" t="inlineStr">
+        <is>
+          <t>{"pump_failure_mode": {"type": "choice", "choice": "bearing", "probabilities": {"seal": 0.004210403841587444, "bearing": 0.9935691479963884, "cavitation": 0.0009314177515951069, "instrument": 0.000396133117015098, "other": 0.0008928972934135872}, "confidence": 0.971844626140937}, "pump_containment": {"type": "noul", "noul": 0.009149884270851874}, "pump_urgency": {"type": "score", "score": 0.01254440492998592, "legend": {"0": "Can wait for the next planned window", "1": "Should be handled within days", "2": "Needs attention now"}, "probabilities": {"0": 0.9895670238896596, "1": 0.008321547290695114, "2": 0.0021114288196454035}, "confidence": 0.942439470709464}}</t>
         </is>
       </c>
     </row>
@@ -16533,7 +19006,12 @@
       </c>
       <c r="B4" s="35" t="inlineStr">
         <is>
-          <t>{"hx_problem": {"type": "choice", "choice": "fouling", "probabilities": {"fouling": 0.9478850419472986, "tube_leak": 0.028015671752445407, "flow_maldistribution": 0.021038713019720476, "control_valve": 0.0009826808054082873, "other": 0.0020778924751272197}, "confidence": 0.8435687329991992}, "hx_crosscontam": {"type": "noul", "noul": 0.02294895360818915}, "hx_impact": {"type": "score", "score": 1.3154958340739715, "legend": {"0": "No noticeable impact", "1": "Reduced duty but operating", "2": "Major loss of duty or unit unusable"}, "probabilities": {"0": 0.10341257644438336, "1": 0.4776790130372617, "2": 0.41890841051835487}, "confidence": 0.13340074156127713}}</t>
+          <t>{"input_tokens": 1104, "output_tokens": 4}</t>
+        </is>
+      </c>
+      <c r="C4" s="35" t="inlineStr">
+        <is>
+          <t>{"hx_problem": {"type": "choice", "choice": "fouling", "probabilities": {"fouling": 0.9479736032978536, "tube_leak": 0.028153284493628594, "flow_maldistribution": 0.020678156580426196, "control_valve": 0.0009853402904680163, "other": 0.0022096153376235015}, "confidence": 0.8436129076949702}, "hx_crosscontam": {"type": "noul", "noul": 0.022169286159840953}, "hx_impact": {"type": "score", "score": 1.300448838097414, "legend": {"0": "No noticeable impact", "1": "Reduced duty but operating", "2": "Major loss of duty or unit unusable"}, "probabilities": {"0": 0.10685025101872331, "1": 0.48585065986513976, "2": 0.40729908911613705}, "confidence": 0.13026238813250735}}</t>
         </is>
       </c>
     </row>
@@ -16545,7 +19023,12 @@
       </c>
       <c r="B5" s="35" t="inlineStr">
         <is>
-          <t>{"hx_problem": {"type": "choice", "choice": "tube_leak", "probabilities": {"fouling": 0.0007413265006967869, "tube_leak": 0.9959796555651736, "flow_maldistribution": 0.00043550090530919514, "control_valve": 0.00032655607260840267, "other": 0.0025169609562122087}, "confidence": 0.9811052724756711}, "hx_crosscontam": {"type": "noul", "noul": 0.9972773611314817}, "hx_impact": {"type": "score", "score": 1.011186618395636, "legend": {"0": "No noticeable impact", "1": "Reduced duty but operating", "2": "Major loss of duty or unit unusable"}, "probabilities": {"0": 0.07036651965596523, "1": 0.8480803422924331, "2": 0.08155313805160146}, "confidence": 0.5167403657884981}}</t>
+          <t>{"input_tokens": 1101, "output_tokens": 4}</t>
+        </is>
+      </c>
+      <c r="C5" s="35" t="inlineStr">
+        <is>
+          <t>{"hx_problem": {"type": "choice", "choice": "tube_leak", "probabilities": {"fouling": 0.0007495941289747238, "tube_leak": 0.9959396543190018, "flow_maldistribution": 0.00044349003446748496, "control_valve": 0.00033230586104586267, "other": 0.0025349556565101997}, "confidence": 0.9809344898041918}, "hx_crosscontam": {"type": "noul", "noul": 0.9973633152102099}, "hx_impact": {"type": "score", "score": 1.0126322136348604, "legend": {"0": "No noticeable impact", "1": "Reduced duty but operating", "2": "Major loss of duty or unit unusable"}, "probabilities": {"0": 0.06982021992433367, "1": 0.8477273465164722, "2": 0.08245243355919417}, "confidence": 0.5160678099489566}}</t>
         </is>
       </c>
     </row>
@@ -16557,7 +19040,12 @@
       </c>
       <c r="B6" s="35" t="inlineStr">
         <is>
-          <t>{"col_symptom": {"type": "choice", "choice": "flooding", "probabilities": {"flooding": 0.5175961061389851, "weeping": 0.012200956102939394, "foaming": 0.4556040469819839, "fouling": 0.001680899310385979, "reboiler_condenser": 0.0013599361901990839, "instrument": 0.010907201436286347, "other": 0.0006508538392200906}, "confidence": 0.575229541784642}, "col_offspec": {"type": "noul", "noul": 0.9990573225259095}, "col_stability": {"type": "score", "score": 1.8194401250687795, "legend": {"0": "Steady operation", "1": "Drifting or minor swings", "2": "Significant upset"}, "probabilities": {"0": 0.07519103740662722, "1": 0.030177800117966076, "2": 0.8946311624754067}, "confidence": 0.6360617217354828}}</t>
+          <t>{"input_tokens": 1185, "output_tokens": 4}</t>
+        </is>
+      </c>
+      <c r="C6" s="35" t="inlineStr">
+        <is>
+          <t>{"col_symptom": {"type": "choice", "choice": "flooding", "probabilities": {"flooding": 0.5213366239870925, "weeping": 0.011961306768748318, "foaming": 0.45219931941914193, "fouling": 0.0016842474743738354, "reboiler_condenser": 0.001308984041366691, "instrument": 0.010858531272865853, "other": 0.0006509870364110156}, "confidence": 0.5761713560101278}, "col_offspec": {"type": "noul", "noul": 0.9990587441403763}, "col_stability": {"type": "score", "score": 1.8190906025969573, "legend": {"0": "Steady operation", "1": "Drifting or minor swings", "2": "Significant upset"}, "probabilities": {"0": 0.07555197936212335, "1": 0.029805438678796, "2": 0.8946425819590806}, "confidence": 0.6363997745790606}}</t>
         </is>
       </c>
     </row>
@@ -16569,7 +19057,12 @@
       </c>
       <c r="B7" s="35" t="inlineStr">
         <is>
-          <t>{"col_symptom": {"type": "choice", "choice": "other", "probabilities": {"flooding": 0.024242860849536994, "weeping": 0.0010585059610439293, "foaming": 0.0006364711561126581, "fouling": 0.0009836821928156953, "reboiler_condenser": 0.00011520558342775971, "instrument": 6.0916933063774306e-05, "other": 0.9729023573239992}, "confidence": 0.9294495624188652}, "col_offspec": {"type": "noul", "noul": 0.0019650654443123363}, "col_stability": {"type": "score", "score": 0.004745121587660906, "legend": {"0": "Steady operation", "1": "Drifting or minor swings", "2": "Significant upset"}, "probabilities": {"0": 0.997151610266207, "1": 0.0009516578799251958, "2": 0.001896731853867855}, "confidence": 0.9805633856279246}}</t>
+          <t>{"input_tokens": 1179, "output_tokens": 4}</t>
+        </is>
+      </c>
+      <c r="C7" s="35" t="inlineStr">
+        <is>
+          <t>{"col_symptom": {"type": "choice", "choice": "other", "probabilities": {"flooding": 0.023605525638543064, "weeping": 0.001033789006631328, "foaming": 0.0006111553689247979, "fouling": 0.0009357907207663385, "reboiler_condenser": 0.00011554811428608701, "instrument": 6.012053392512738e-05, "other": 0.9736380706169232}, "confidence": 0.9310185171064398}, "col_offspec": {"type": "noul", "noul": 0.002046953021448908}, "col_stability": {"type": "score", "score": 0.004613240175433055, "legend": {"0": "Steady operation", "1": "Drifting or minor swings", "2": "Significant upset"}, "probabilities": {"0": 0.9972211021457282, "1": 0.0009445555331100775, "2": 0.0018343423211614886}, "confidence": 0.980965088363793}}</t>
         </is>
       </c>
     </row>
@@ -16678,7 +19171,7 @@
         <v>0</v>
       </c>
       <c r="F2" s="35" t="n">
-        <v>0.928</v>
+        <v>0.929</v>
       </c>
       <c r="G2" s="35" t="n">
         <v>2</v>
@@ -16690,7 +19183,7 @@
         <v>1</v>
       </c>
       <c r="J2" s="35" t="n">
-        <v>0.928</v>
+        <v>0.929</v>
       </c>
       <c r="K2" s="35" t="inlineStr"/>
     </row>
@@ -16752,7 +19245,7 @@
         <v>1</v>
       </c>
       <c r="F4" s="35" t="n">
-        <v>0.726</v>
+        <v>0.728</v>
       </c>
       <c r="G4" s="35" t="n">
         <v>2</v>
@@ -16764,7 +19257,7 @@
         <v>1</v>
       </c>
       <c r="J4" s="35" t="n">
-        <v>0.726</v>
+        <v>0.728</v>
       </c>
       <c r="K4" s="35" t="inlineStr"/>
     </row>
@@ -16826,7 +19319,7 @@
         <v>0</v>
       </c>
       <c r="F6" s="35" t="n">
-        <v>0.987</v>
+        <v>0.988</v>
       </c>
       <c r="G6" s="35" t="n">
         <v>2</v>
@@ -16838,7 +19331,7 @@
         <v>1</v>
       </c>
       <c r="J6" s="35" t="n">
-        <v>0.987</v>
+        <v>0.988</v>
       </c>
       <c r="K6" s="35" t="inlineStr"/>
     </row>
@@ -16863,7 +19356,7 @@
         <v>2</v>
       </c>
       <c r="F7" s="35" t="n">
-        <v>0.325</v>
+        <v>0.323</v>
       </c>
       <c r="G7" s="35" t="n">
         <v>2</v>
@@ -16875,10 +19368,10 @@
         <v>0.5</v>
       </c>
       <c r="J7" s="35" t="n">
-        <v>0.133</v>
+        <v>0.13</v>
       </c>
       <c r="K7" s="35" t="n">
-        <v>0.517</v>
+        <v>0.516</v>
       </c>
     </row>
     <row r="8">
@@ -16902,7 +19395,7 @@
         <v>1</v>
       </c>
       <c r="F8" s="35" t="n">
-        <v>0.752</v>
+        <v>0.754</v>
       </c>
       <c r="G8" s="35" t="n">
         <v>2</v>
@@ -16914,7 +19407,7 @@
         <v>1</v>
       </c>
       <c r="J8" s="35" t="n">
-        <v>0.752</v>
+        <v>0.754</v>
       </c>
       <c r="K8" s="35" t="inlineStr"/>
     </row>
@@ -16976,7 +19469,7 @@
         <v>0</v>
       </c>
       <c r="F10" s="35" t="n">
-        <v>0.8080000000000001</v>
+        <v>0.8090000000000001</v>
       </c>
       <c r="G10" s="35" t="n">
         <v>2</v>
@@ -16988,7 +19481,7 @@
         <v>1</v>
       </c>
       <c r="J10" s="35" t="n">
-        <v>0.8080000000000001</v>
+        <v>0.8090000000000001</v>
       </c>
       <c r="K10" s="35" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Refresh workbook outputs from clean dual-engine QC rerun.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/nimble_classifier_workbook.xlsx
+++ b/nimble_classifier_workbook.xlsx
@@ -920,7 +920,7 @@
       </c>
       <c r="B2" s="35" t="inlineStr">
         <is>
-          <t>20260930_142141</t>
+          <t>20260930_142515</t>
         </is>
       </c>
     </row>
@@ -1064,7 +1064,7 @@
       </c>
       <c r="B14" s="35" t="inlineStr">
         <is>
-          <t>45.3</t>
+          <t>5.1</t>
         </is>
       </c>
     </row>
@@ -1076,7 +1076,7 @@
       </c>
       <c r="B15" s="35" t="inlineStr">
         <is>
-          <t>/mnt/d/dev/nimble_plant/nimble_classifier_workbook_nimble_20260930_142141.jsonl</t>
+          <t>/mnt/d/dev/nimble_plant/nimble_classifier_workbook_nimble_20260930_142515.jsonl</t>
         </is>
       </c>
     </row>
@@ -1400,10 +1400,10 @@
         </is>
       </c>
       <c r="I2" s="37" t="n">
-        <v>0.9</v>
+        <v>0.89</v>
       </c>
       <c r="J2" s="37" t="n">
-        <v>0.9</v>
+        <v>0.89</v>
       </c>
       <c r="K2" s="35" t="inlineStr">
         <is>
@@ -1565,10 +1565,10 @@
         </is>
       </c>
       <c r="R4" s="37" t="n">
-        <v>0.87</v>
+        <v>0.86</v>
       </c>
       <c r="S4" s="37" t="n">
-        <v>0.13</v>
+        <v>0.14</v>
       </c>
       <c r="T4" s="35" t="inlineStr">
         <is>
@@ -1576,10 +1576,10 @@
         </is>
       </c>
       <c r="U4" s="37" t="n">
-        <v>0.86</v>
+        <v>0.84</v>
       </c>
       <c r="V4" s="37" t="n">
-        <v>1.09</v>
+        <v>1.1</v>
       </c>
       <c r="W4" s="35" t="inlineStr"/>
       <c r="X4" s="35" t="inlineStr"/>
@@ -1657,7 +1657,7 @@
         <v>0.49</v>
       </c>
       <c r="V5" s="34" t="n">
-        <v>1.27</v>
+        <v>1.25</v>
       </c>
       <c r="W5" s="32" t="inlineStr"/>
       <c r="X5" s="32" t="inlineStr"/>
@@ -1723,10 +1723,10 @@
         </is>
       </c>
       <c r="X6" s="37" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.84</v>
       </c>
       <c r="Y6" s="37" t="n">
-        <v>0.84</v>
+        <v>0.87</v>
       </c>
       <c r="Z6" s="35" t="inlineStr">
         <is>
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C2" s="35" t="inlineStr">
         <is>
-          <t>{"pump_failure_mode": {"type": "choice", "choice": "seal", "confidence": 1.0, "probabilities": {"cavitation": 0.0, "bearing": 0.0, "instrument": 0.0, "seal": 1.0, "other": 0.0}}, "pump_containment": {"type": "noul", "noul": 0.9}, "pump_urgency": {"type": "score", "score": 1.99, "confidence": 0.99, "legend": {"0": "Can wait for the next planned window", "1": "Should be handled within days", "2": "Needs attention now"}, "probabilities": {"0": 0.0, "1": 0.01, "2": 0.99}}}</t>
+          <t>{"pump_failure_mode": {"type": "choice", "choice": "seal", "confidence": 1.0, "probabilities": {"cavitation": 0.0, "bearing": 0.0, "instrument": 0.0, "seal": 1.0, "other": 0.0}}, "pump_containment": {"type": "noul", "noul": 0.89}, "pump_urgency": {"type": "score", "score": 1.99, "confidence": 0.99, "legend": {"0": "Can wait for the next planned window", "1": "Should be handled within days", "2": "Needs attention now"}, "probabilities": {"0": 0.0, "1": 0.01, "2": 0.99}}}</t>
         </is>
       </c>
     </row>
@@ -1900,7 +1900,7 @@
       </c>
       <c r="C3" s="35" t="inlineStr">
         <is>
-          <t>{"pump_failure_mode": {"type": "choice", "choice": "bearing", "confidence": 1.0, "probabilities": {"instrument": 0.0, "other": 0.0, "cavitation": 0.0, "seal": 0.0, "bearing": 1.0}}, "pump_containment": {"type": "noul", "noul": 0.01}, "pump_urgency": {"type": "score", "score": 0.01, "confidence": 0.99, "legend": {"0": "Can wait for the next planned window", "1": "Should be handled within days", "2": "Needs attention now"}, "probabilities": {"0": 0.99, "1": 0.01, "2": 0.0}}}</t>
+          <t>{"pump_failure_mode": {"type": "choice", "choice": "bearing", "confidence": 1.0, "probabilities": {"other": 0.0, "seal": 0.0, "cavitation": 0.0, "bearing": 1.0, "instrument": 0.0}}, "pump_containment": {"type": "noul", "noul": 0.01}, "pump_urgency": {"type": "score", "score": 0.01, "confidence": 0.99, "legend": {"0": "Can wait for the next planned window", "1": "Should be handled within days", "2": "Needs attention now"}, "probabilities": {"0": 1.0, "1": 0.0, "2": 0.0}}}</t>
         </is>
       </c>
     </row>
@@ -1917,7 +1917,7 @@
       </c>
       <c r="C4" s="35" t="inlineStr">
         <is>
-          <t>{"hx_problem": {"type": "choice", "choice": "fouling", "confidence": 1.0, "probabilities": {"tube_leak": 0.0, "other": 0.0, "flow_maldistribution": 0.0, "control_valve": 0.0, "fouling": 1.0}}, "hx_crosscontam": {"type": "noul", "noul": 0.13}, "hx_impact": {"type": "score", "score": 1.09, "confidence": 0.86, "legend": {"0": "No noticeable impact", "1": "Reduced duty but operating", "2": "Major loss of duty or unit unusable"}, "probabilities": {"0": 0.0, "1": 0.91, "2": 0.09}}}</t>
+          <t>{"hx_problem": {"type": "choice", "choice": "fouling", "confidence": 1.0, "probabilities": {"control_valve": 0.0, "tube_leak": 0.0, "other": 0.0, "flow_maldistribution": 0.0, "fouling": 1.0}}, "hx_crosscontam": {"type": "noul", "noul": 0.14}, "hx_impact": {"type": "score", "score": 1.1, "confidence": 0.84, "legend": {"0": "No noticeable impact", "1": "Reduced duty but operating", "2": "Major loss of duty or unit unusable"}, "probabilities": {"0": 0.0, "1": 0.9, "2": 0.1}}}</t>
         </is>
       </c>
     </row>
@@ -1934,7 +1934,7 @@
       </c>
       <c r="C5" s="35" t="inlineStr">
         <is>
-          <t>{"hx_problem": {"type": "choice", "choice": "tube_leak", "confidence": 1.0, "probabilities": {"other": 0.0, "fouling": 0.0, "flow_maldistribution": 0.0, "tube_leak": 1.0, "control_valve": 0.0}}, "hx_crosscontam": {"type": "noul", "noul": 0.9}, "hx_impact": {"type": "score", "score": 1.27, "confidence": 0.49, "legend": {"0": "No noticeable impact", "1": "Reduced duty but operating", "2": "Major loss of duty or unit unusable"}, "probabilities": {"0": 0.04, "1": 0.66, "2": 0.3}}}</t>
+          <t>{"hx_problem": {"type": "choice", "choice": "tube_leak", "confidence": 1.0, "probabilities": {"control_valve": 0.0, "flow_maldistribution": 0.0, "other": 0.0, "tube_leak": 1.0, "fouling": 0.0}}, "hx_crosscontam": {"type": "noul", "noul": 0.9}, "hx_impact": {"type": "score", "score": 1.25, "confidence": 0.49, "legend": {"0": "No noticeable impact", "1": "Reduced duty but operating", "2": "Major loss of duty or unit unusable"}, "probabilities": {"0": 0.05, "1": 0.65, "2": 0.3}}}</t>
         </is>
       </c>
     </row>
@@ -1951,7 +1951,7 @@
       </c>
       <c r="C6" s="35" t="inlineStr">
         <is>
-          <t>{"col_symptom": {"type": "choice", "choice": "flooding", "confidence": 0.81, "probabilities": {"flooding": 0.84, "foaming": 0.08, "fouling": 0.01, "weeping": 0.0, "instrument": 0.04, "other": 0.03, "reboiler_condenser": 0.0}}, "col_offspec": {"type": "noul", "noul": 0.99}, "col_stability": {"type": "score", "score": 2.0, "confidence": 1.0, "legend": {"0": "Steady operation", "1": "Drifting or minor swings", "2": "Significant upset"}, "probabilities": {"0": 0.0, "1": 0.0, "2": 1.0}}}</t>
+          <t>{"col_symptom": {"type": "choice", "choice": "flooding", "confidence": 0.84, "probabilities": {"instrument": 0.02, "flooding": 0.87, "other": 0.02, "reboiler_condenser": 0.0, "weeping": 0.0, "foaming": 0.09, "fouling": 0.0}}, "col_offspec": {"type": "noul", "noul": 0.99}, "col_stability": {"type": "score", "score": 2.0, "confidence": 1.0, "legend": {"0": "Steady operation", "1": "Drifting or minor swings", "2": "Significant upset"}, "probabilities": {"0": 0.0, "1": 0.0, "2": 1.0}}}</t>
         </is>
       </c>
     </row>
@@ -1968,7 +1968,7 @@
       </c>
       <c r="C7" s="35" t="inlineStr">
         <is>
-          <t>{"col_symptom": {"type": "choice", "choice": "other", "confidence": 1.0, "probabilities": {"weeping": 0.0, "instrument": 0.0, "foaming": 0.0, "flooding": 0.0, "reboiler_condenser": 0.0, "fouling": 0.0, "other": 1.0}}, "col_offspec": {"type": "noul", "noul": 0.01}, "col_stability": {"type": "score", "score": 0.0, "confidence": 1.0, "legend": {"0": "Steady operation", "1": "Drifting or minor swings", "2": "Significant upset"}, "probabilities": {"0": 1.0, "1": 0.0, "2": 0.0}}}</t>
+          <t>{"col_symptom": {"type": "choice", "choice": "other", "confidence": 1.0, "probabilities": {"fouling": 0.0, "weeping": 0.0, "other": 1.0, "flooding": 0.0, "foaming": 0.0, "reboiler_condenser": 0.0, "instrument": 0.0}}, "col_offspec": {"type": "noul", "noul": 0.01}, "col_stability": {"type": "score", "score": 0.0, "confidence": 1.0, "legend": {"0": "Steady operation", "1": "Drifting or minor swings", "2": "Significant upset"}, "probabilities": {"0": 1.0, "1": 0.0, "2": 0.0}}}</t>
         </is>
       </c>
     </row>
@@ -2114,7 +2114,7 @@
         <v>0</v>
       </c>
       <c r="F3" s="35" t="n">
-        <v>0.945</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="G3" s="35" t="n">
         <v>2</v>
@@ -2126,7 +2126,7 @@
         <v>1</v>
       </c>
       <c r="J3" s="35" t="n">
-        <v>0.945</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="K3" s="35" t="inlineStr"/>
     </row>
@@ -2225,7 +2225,7 @@
         <v>0</v>
       </c>
       <c r="F6" s="35" t="n">
-        <v>0.885</v>
+        <v>0.88</v>
       </c>
       <c r="G6" s="35" t="n">
         <v>2</v>
@@ -2237,7 +2237,7 @@
         <v>1</v>
       </c>
       <c r="J6" s="35" t="n">
-        <v>0.885</v>
+        <v>0.88</v>
       </c>
       <c r="K6" s="35" t="inlineStr"/>
     </row>
@@ -2262,7 +2262,7 @@
         <v>1</v>
       </c>
       <c r="F7" s="35" t="n">
-        <v>0.675</v>
+        <v>0.665</v>
       </c>
       <c r="G7" s="35" t="n">
         <v>2</v>
@@ -2274,7 +2274,7 @@
         <v>0.5</v>
       </c>
       <c r="J7" s="35" t="n">
-        <v>0.86</v>
+        <v>0.84</v>
       </c>
       <c r="K7" s="35" t="n">
         <v>0.49</v>
@@ -2301,7 +2301,7 @@
         <v>0</v>
       </c>
       <c r="F8" s="35" t="n">
-        <v>0.905</v>
+        <v>0.92</v>
       </c>
       <c r="G8" s="35" t="n">
         <v>2</v>
@@ -2313,7 +2313,7 @@
         <v>1</v>
       </c>
       <c r="J8" s="35" t="n">
-        <v>0.905</v>
+        <v>0.92</v>
       </c>
       <c r="K8" s="35" t="inlineStr"/>
     </row>
@@ -2429,7 +2429,7 @@
       </c>
       <c r="B2" s="35" t="inlineStr">
         <is>
-          <t>20260930_142230</t>
+          <t>20260930_142521</t>
         </is>
       </c>
     </row>
@@ -2585,7 +2585,7 @@
       </c>
       <c r="B15" s="35" t="inlineStr">
         <is>
-          <t>/mnt/d/dev/nimble_plant/nimble_classifier_workbook_jev_20260930_142230.jsonl</t>
+          <t>/mnt/d/dev/nimble_plant/nimble_classifier_workbook_jev_20260930_142521.jsonl</t>
         </is>
       </c>
     </row>
@@ -2755,7 +2755,7 @@
         <v>0.9347743692709441</v>
       </c>
       <c r="G2" s="35" t="n">
-        <v>0.9</v>
+        <v>0.89</v>
       </c>
       <c r="H2" s="35" t="inlineStr">
         <is>
@@ -3007,7 +3007,7 @@
         <v>0.9778307138401591</v>
       </c>
       <c r="G8" s="35" t="n">
-        <v>0.87</v>
+        <v>0.86</v>
       </c>
       <c r="H8" s="35" t="inlineStr">
         <is>
@@ -3049,7 +3049,7 @@
         <v>0.1302623881325073</v>
       </c>
       <c r="G9" s="35" t="n">
-        <v>0.86</v>
+        <v>0.84</v>
       </c>
       <c r="H9" s="35" t="inlineStr">
         <is>
@@ -3343,7 +3343,7 @@
         <v>0.5761713560101278</v>
       </c>
       <c r="G16" s="35" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.84</v>
       </c>
       <c r="H16" s="35" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Clean up documentation set for v1.0-dev.
Align README, functional spec, experiments archive note, runner docstring, and workbook Read Me; add docs index.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/nimble_classifier_workbook.xlsx
+++ b/nimble_classifier_workbook.xlsx
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="28" customWidth="1" style="16" min="1" max="1"/>
@@ -634,246 +634,269 @@
     <row r="1" ht="17.35" customHeight="1" s="17">
       <c r="A1" s="46" t="inlineStr">
         <is>
-          <t>Nimble / Jev batch classifier - control workbook</t>
+          <t>Nimble / Jev batch classifier — control workbook (v1.0-dev)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" s="17">
-      <c r="A2" s="16" t="inlineStr">
-        <is>
-          <t>Define questions, labels and records here. Run with --engine nimble or --engine jev. Each engine writes its own output_&lt;engine&gt;_* sheets and does not clear the other. When both Results sheets exist, output_compare is refreshed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="17">
-      <c r="A4" s="16" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Edit questions, labels, and records here. Run: python nimble_runner.py &lt;this file&gt; --engine nimble|jev. Each engine writes output_&lt;engine&gt;_* only and does not clear the other. When both Results sheets exist, output_compare is refreshed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Docs: repo README.md (quick start); docs/functional-spec.md (as-built spec + UML).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="17"/>
+    <row r="5" ht="15" customHeight="1" s="17">
+      <c r="A5" t="inlineStr">
         <is>
           <t>SHEETS</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="17">
-      <c r="A5" s="16" t="inlineStr">
+    <row r="6" ht="30" customHeight="1" s="17">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Config</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
-        <is>
-          <t>Settings: engine (nimble|jev), timeouts, review threshold, test-run size. Engine preset overrides model/base_url/endpoint.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1" s="17">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>engine (nimble|jev), timeouts, review threshold, test_first_n. Runtime preset overrides model/base_url/endpoint.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1" s="17">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Questions</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>One row per question. Type is choice, noul (yes/no) or score. Leave equipment_type blank to ask every record.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1" s="17">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>One row per question: choice, noul (yes/no), or score. Blank equipment_type = all records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1" s="17">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Labels</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
-        <is>
-          <t>Answer options for choice and score only. For score, order is scale position (lowest first).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1" s="17">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Options for choice and score only. For score, order is scale position (lowest first).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1" s="17">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Records</t>
         </is>
       </c>
-      <c r="B8" s="16" t="inlineStr">
-        <is>
-          <t>Statements to classify. Optional expected_&lt;question_id&gt; columns for accuracy.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="17">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Text to classify. Optional expected_&lt;question_id&gt; for accuracy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1" s="17">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Lists</t>
         </is>
       </c>
-      <c r="B9" s="16" t="inlineStr">
-        <is>
-          <t>Dropdown values (equipment types).</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="17">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Equipment-type dropdown values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1" s="17">
+      <c r="A11" t="inlineStr">
         <is>
           <t>output_nimble_*</t>
         </is>
       </c>
-      <c r="B10" s="16" t="inlineStr">
-        <is>
-          <t>Written by --engine nimble: Results, Raw, Summary, Run_info.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1" s="17">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Results / Raw / Summary / Run_info from --engine nimble.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1" s="17">
+      <c r="A12" t="inlineStr">
         <is>
           <t>output_jev_*</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
-        <is>
-          <t>Written by --engine jev: Results, Raw, Summary, Run_info.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="15" customHeight="1" s="17">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Results / Raw / Summary / Run_info from --engine jev.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1" s="17">
+      <c r="A13" t="inlineStr">
         <is>
           <t>output_compare</t>
         </is>
       </c>
-      <c r="B12" s="16" t="inlineStr">
-        <is>
-          <t>Side-by-side Nimble vs Jev answers when both Results sheets exist. Diffs highlighted.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="15" customHeight="1" s="17">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Nimble vs Jev answers when both Results exist. Diffs highlighted orange.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="45" customHeight="1" s="17"/>
+    <row r="15" ht="30" customHeight="1" s="17">
+      <c r="A15" t="inlineStr">
         <is>
           <t>COLOURS</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="45" customHeight="1" s="17">
-      <c r="A14" s="16" t="inlineStr">
+    <row r="16" ht="15" customHeight="1" s="17">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Blue text</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
-        <is>
-          <t>Cells you edit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1" s="17">
-      <c r="A15" s="16" t="inlineStr">
-        <is>
-          <t>Black text, grey fill</t>
-        </is>
-      </c>
-      <c r="B15" s="16" t="inlineStr">
-        <is>
-          <t>Formulas. Do not edit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="15" customHeight="1" s="17">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Editable cells.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1" s="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Grey fill / formulas</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Do not edit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1" s="17">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Yellow row</t>
         </is>
       </c>
-      <c r="B16" s="16" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Flagged for review (low confidence).</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="30" customHeight="1" s="17">
-      <c r="A17" s="16" t="inlineStr">
+    <row r="19" ht="30" customHeight="1" s="17">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Orange row (compare)</t>
         </is>
       </c>
-      <c r="B17" s="16" t="inlineStr">
-        <is>
-          <t>Nimble and Jev answers disagree.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1" s="17">
-      <c r="A18" s="16" t="inlineStr">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Engines disagree.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1" s="17"/>
+    <row r="21" ht="45" customHeight="1" s="17">
+      <c r="A21" t="inlineStr">
         <is>
           <t>RULES</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="30" customHeight="1" s="17">
-      <c r="A19" s="16" t="inlineStr">
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>Engine</t>
         </is>
       </c>
-      <c r="B19" s="16" t="inlineStr">
-        <is>
-          <t>Use Config engine or CLI --engine. Jev needs TYPESAFE_API_KEY. Nimble needs local Ollama &gt;= 0.35.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="15" customHeight="1" s="17">
-      <c r="A20" s="16" t="inlineStr">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Config engine or CLI --engine. Nimble: Ollama &gt;= 0.35. Jev: export TYPESAFE_API_KEY (leave Config api_key blank).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>IDs</t>
         </is>
       </c>
-      <c r="B20" s="16" t="inlineStr">
-        <is>
-          <t>question_id and label: short lowercase with underscores, no spaces.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="45" customHeight="1" s="17">
-      <c r="A21" s="16" t="inlineStr">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>question_id and label: letters, digits, _ or -; no spaces.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>Always add 'other'</t>
         </is>
       </c>
-      <c r="B21" s="16" t="inlineStr">
-        <is>
-          <t>Include other on every choice question.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="16" t="inlineStr">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>On every choice question so vague text is not forced into a wrong label.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>Expected values</t>
         </is>
       </c>
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>choice: a Labels value; noul: true or false.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="16" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Close workbook</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Unlock/close this file in Excel/LibreOffice before running the classifier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27"/>
+    <row r="28">
+      <c r="A28" t="inlineStr">
         <is>
           <t>EXAMPLES</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="16" t="inlineStr">
+    <row r="29">
+      <c r="A29" t="inlineStr">
         <is>
           <t>Example rows</t>
         </is>
       </c>
-      <c r="B24" s="16" t="inlineStr">
-        <is>
-          <t>Illustrative pumps / exchangers / columns. Replace with your plant data.</t>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Illustrative pumps / exchangers / columns — replace with plant data.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rewrite README for Nimble and Jev; remove extra docs README.
One clear operator guide at the root; archive note and workbook Read Me aligned to the same story.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/nimble_classifier_workbook.xlsx
+++ b/nimble_classifier_workbook.xlsx
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="28" customWidth="1" style="16" min="1" max="1"/>
@@ -634,269 +634,296 @@
     <row r="1" ht="17.35" customHeight="1" s="17">
       <c r="A1" s="46" t="inlineStr">
         <is>
-          <t>Nimble / Jev batch classifier — control workbook (v1.0-dev)</t>
+          <t>Nimble and Jev — control workbook</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" s="17">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Edit questions, labels, and records here. Run: python nimble_runner.py &lt;this file&gt; --engine nimble|jev. Each engine writes output_&lt;engine&gt;_* only and does not clear the other. When both Results sheets exist, output_compare is refreshed.</t>
+          <t>This one workbook works with BOTH engines: Nimble (local Ollama) and Jev (TypeSafe cloud).</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Docs: repo README.md (quick start); docs/functional-spec.md (as-built spec + UML).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="17"/>
-    <row r="5" ht="15" customHeight="1" s="17">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>SHEETS</t>
-        </is>
-      </c>
-    </row>
+          <t>Edit questions and records here. Run from the terminal (see the repo README.md). Use --engine nimble or --engine jev.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="17">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Each engine writes its own output_&lt;engine&gt;_* sheets and does not clear the other. When both Results exist, output_compare is filled in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1" s="17"/>
     <row r="6" ht="30" customHeight="1" s="17">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Config</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>engine (nimble|jev), timeouts, review threshold, test_first_n. Runtime preset overrides model/base_url/endpoint.</t>
+          <t>SHEETS YOU EDIT</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" s="17">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Questions</t>
+          <t>Config</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>One row per question: choice, noul (yes/no), or score. Blank equipment_type = all records.</t>
+          <t>Default engine, timeouts, review threshold, test size. Runtime preset still sets model/URL for the chosen engine.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1" s="17">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Labels</t>
+          <t>Questions</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Options for choice and score only. For score, order is scale position (lowest first).</t>
+          <t>One row per question: choice, noul (yes/no), or score. Blank equipment_type = ask every record.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="17">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Records</t>
+          <t>Labels</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Text to classify. Optional expected_&lt;question_id&gt; for accuracy.</t>
+          <t>Options for choice and score only. For score, order is the scale (lowest first).</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="17">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Lists</t>
+          <t>Records</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Equipment-type dropdown values.</t>
+          <t>Text to classify. Optional expected_&lt;question_id&gt; for accuracy checks.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="17">
       <c r="A11" t="inlineStr">
         <is>
-          <t>output_nimble_*</t>
+          <t>Lists</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Results / Raw / Summary / Run_info from --engine nimble.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="15" customHeight="1" s="17">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>output_jev_*</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Results / Raw / Summary / Run_info from --engine jev.</t>
-        </is>
-      </c>
-    </row>
+          <t>Equipment-type dropdown values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1" s="17"/>
     <row r="13" ht="15" customHeight="1" s="17">
       <c r="A13" t="inlineStr">
         <is>
-          <t>output_compare</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Nimble vs Jev answers when both Results exist. Diffs highlighted orange.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="45" customHeight="1" s="17"/>
+          <t>SHEETS THE RUNNER WRITES</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="45" customHeight="1" s="17">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>output_nimble_*</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Results / Raw / Summary / Run_info from a Nimble run.</t>
+        </is>
+      </c>
+    </row>
     <row r="15" ht="30" customHeight="1" s="17">
       <c r="A15" t="inlineStr">
         <is>
-          <t>COLOURS</t>
+          <t>output_jev_*</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Results / Raw / Summary / Run_info from a Jev run.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="17">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Blue text</t>
+          <t>output_compare</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Editable cells.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1" s="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Grey fill / formulas</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Do not edit.</t>
-        </is>
-      </c>
-    </row>
+          <t>Side-by-side Nimble vs Jev when both Results sheets exist. Diffs highlighted orange.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1" s="17"/>
     <row r="18" ht="30" customHeight="1" s="17">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Yellow row</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Flagged for review (low confidence).</t>
+          <t>COLOURS</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1" s="17">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Orange row (compare)</t>
+          <t>Blue text</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Engines disagree.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="15" customHeight="1" s="17"/>
+          <t>Editable cells.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1" s="17">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Grey fill / formulas</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Do not edit.</t>
+        </is>
+      </c>
+    </row>
     <row r="21" ht="45" customHeight="1" s="17">
       <c r="A21" t="inlineStr">
         <is>
-          <t>RULES</t>
+          <t>Yellow row</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Flagged for review (low confidence).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Engine</t>
+          <t>Orange row (compare)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Config engine or CLI --engine. Nimble: Ollama &gt;= 0.35. Jev: export TYPESAFE_API_KEY (leave Config api_key blank).</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>IDs</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>question_id and label: letters, digits, _ or -; no spaces.</t>
-        </is>
-      </c>
-    </row>
+          <t>Nimble and Jev disagree.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Always add 'other'</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>On every choice question so vague text is not forced into a wrong label.</t>
+          <t>RULES</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Expected values</t>
+          <t>How to run</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>choice: a Labels value; noul: true or false.</t>
+          <t>Commands are in the repo README.md — not inside this spreadsheet.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Close workbook</t>
+          <t>Engine</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Unlock/close this file in Excel/LibreOffice before running the classifier.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27"/>
+          <t>Config engine or CLI --engine. Nimble needs Ollama &gt;= 0.35. Jev needs TYPESAFE_API_KEY in the environment (leave Config api_key blank).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>IDs</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>question_id and label: letters, digits, _ or -; no spaces.</t>
+        </is>
+      </c>
+    </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>EXAMPLES</t>
+          <t>Always add 'other'</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>On every choice question so vague text is not forced into a wrong label.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>Expected values</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>choice: a Labels value; noul: true or false.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Close workbook</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Close this file in Excel/LibreOffice before running the classifier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31"/>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>EXAMPLES</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>Example rows</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Illustrative pumps / exchangers / columns — replace with plant data.</t>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Illustrative pumps / exchangers / columns — replace with your plant data.</t>
         </is>
       </c>
     </row>

</xml_diff>